<commit_message>
Check left-right confusion separately, mostly same failures as far-away misses
</commit_message>
<xml_diff>
--- a/result/tables/vertebra_anchored_shoulder.xlsx
+++ b/result/tables/vertebra_anchored_shoulder.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N81"/>
+  <dimension ref="A1:Q81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,50 +440,65 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>height</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>banded</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>vert_x</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>vert_y</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>match_score</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>peak_margin</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>near_exact_fraction</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>mae</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>rmse</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>ssim</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>pearson_corr</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>hist_intersection</t>
         </is>
@@ -504,34 +519,43 @@
       <c r="D2" t="n">
         <v>175</v>
       </c>
-      <c r="E2" t="b">
-        <v>1</v>
+      <c r="E2" t="n">
+        <v>90</v>
       </c>
       <c r="F2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="I2" t="n">
         <v>163</v>
       </c>
-      <c r="G2" t="n">
+      <c r="J2" t="n">
         <v>0.5385264158248901</v>
       </c>
-      <c r="H2" t="n">
+      <c r="K2" t="n">
         <v>0.04935389757156372</v>
       </c>
-      <c r="I2" t="n">
+      <c r="L2" t="n">
         <v>0.3171296296296297</v>
       </c>
-      <c r="J2" t="n">
+      <c r="M2" t="n">
         <v>5.95775462962963</v>
       </c>
-      <c r="K2" t="n">
+      <c r="N2" t="n">
         <v>8.229667706265882</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O2" t="n">
         <v>0.6144105734822799</v>
       </c>
-      <c r="M2" t="n">
+      <c r="P2" t="n">
         <v>0.5385264075493138</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Q2" t="n">
         <v>0.4670138888888889</v>
       </c>
     </row>
@@ -550,34 +574,43 @@
       <c r="D3" t="n">
         <v>174</v>
       </c>
-      <c r="E3" t="b">
-        <v>1</v>
+      <c r="E3" t="n">
+        <v>92</v>
       </c>
       <c r="F3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="I3" t="n">
         <v>163</v>
       </c>
-      <c r="G3" t="n">
+      <c r="J3" t="n">
         <v>0.5939807295799255</v>
       </c>
-      <c r="H3" t="n">
+      <c r="K3" t="n">
         <v>0.1391007602214813</v>
       </c>
-      <c r="I3" t="n">
+      <c r="L3" t="n">
         <v>0.3074517978113601</v>
       </c>
-      <c r="J3" t="n">
+      <c r="M3" t="n">
         <v>5.562793121417405</v>
       </c>
-      <c r="K3" t="n">
+      <c r="N3" t="n">
         <v>7.240130476542034</v>
       </c>
-      <c r="L3" t="n">
+      <c r="O3" t="n">
         <v>0.61934347089055</v>
       </c>
-      <c r="M3" t="n">
+      <c r="P3" t="n">
         <v>0.5939807008846184</v>
       </c>
-      <c r="N3" t="n">
+      <c r="Q3" t="n">
         <v>0.4684731631057842</v>
       </c>
     </row>
@@ -596,34 +629,43 @@
       <c r="D4" t="n">
         <v>179</v>
       </c>
-      <c r="E4" t="b">
-        <v>1</v>
+      <c r="E4" t="n">
+        <v>88</v>
       </c>
       <c r="F4" t="n">
+        <v>33</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>129</v>
+      </c>
+      <c r="I4" t="n">
         <v>171</v>
       </c>
-      <c r="G4" t="n">
+      <c r="J4" t="n">
         <v>0.5818588137626648</v>
       </c>
-      <c r="H4" t="n">
+      <c r="K4" t="n">
         <v>0.03272014856338501</v>
       </c>
-      <c r="I4" t="n">
+      <c r="L4" t="n">
         <v>0.2537517053206003</v>
       </c>
-      <c r="J4" t="n">
+      <c r="M4" t="n">
         <v>5.28581173260573</v>
       </c>
-      <c r="K4" t="n">
+      <c r="N4" t="n">
         <v>6.642960351935018</v>
       </c>
-      <c r="L4" t="n">
+      <c r="O4" t="n">
         <v>0.4645026812799135</v>
       </c>
-      <c r="M4" t="n">
+      <c r="P4" t="n">
         <v>0.5818587987158285</v>
       </c>
-      <c r="N4" t="n">
+      <c r="Q4" t="n">
         <v>0.4768076398362892</v>
       </c>
     </row>
@@ -642,34 +684,43 @@
       <c r="D5" t="n">
         <v>186</v>
       </c>
-      <c r="E5" t="b">
-        <v>1</v>
+      <c r="E5" t="n">
+        <v>95</v>
       </c>
       <c r="F5" t="n">
+        <v>43</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>129</v>
+      </c>
+      <c r="I5" t="n">
         <v>171</v>
       </c>
-      <c r="G5" t="n">
+      <c r="J5" t="n">
         <v>0.5113841891288757</v>
       </c>
-      <c r="H5" t="n">
+      <c r="K5" t="n">
         <v>0.1100369691848755</v>
       </c>
-      <c r="I5" t="n">
+      <c r="L5" t="n">
         <v>0.2682512733446519</v>
       </c>
-      <c r="J5" t="n">
+      <c r="M5" t="n">
         <v>5.685483870967742</v>
       </c>
-      <c r="K5" t="n">
+      <c r="N5" t="n">
         <v>7.444503219380164</v>
       </c>
-      <c r="L5" t="n">
+      <c r="O5" t="n">
         <v>0.4976518155727505</v>
       </c>
-      <c r="M5" t="n">
+      <c r="P5" t="n">
         <v>0.5113842093786981</v>
       </c>
-      <c r="N5" t="n">
+      <c r="Q5" t="n">
         <v>0.4936332767402377</v>
       </c>
     </row>
@@ -688,34 +739,43 @@
       <c r="D6" t="n">
         <v>137</v>
       </c>
-      <c r="E6" t="b">
-        <v>1</v>
+      <c r="E6" t="n">
+        <v>71</v>
       </c>
       <c r="F6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="I6" t="n">
         <v>120</v>
       </c>
-      <c r="G6" t="n">
+      <c r="J6" t="n">
         <v>0.9212394952774048</v>
       </c>
-      <c r="H6" t="n">
+      <c r="K6" t="n">
         <v>0.08853447437286377</v>
       </c>
-      <c r="I6" t="n">
+      <c r="L6" t="n">
         <v>0.1865222623345367</v>
       </c>
-      <c r="J6" t="n">
+      <c r="M6" t="n">
         <v>13.1841155234657</v>
       </c>
-      <c r="K6" t="n">
+      <c r="N6" t="n">
         <v>20.53455307612272</v>
       </c>
-      <c r="L6" t="n">
+      <c r="O6" t="n">
         <v>0.8236815706314243</v>
       </c>
-      <c r="M6" t="n">
+      <c r="P6" t="n">
         <v>0.9212394849529599</v>
       </c>
-      <c r="N6" t="n">
+      <c r="Q6" t="n">
         <v>0.6221419975932612</v>
       </c>
     </row>
@@ -734,34 +794,43 @@
       <c r="D7" t="n">
         <v>114</v>
       </c>
-      <c r="E7" t="b">
-        <v>1</v>
+      <c r="E7" t="n">
+        <v>86</v>
       </c>
       <c r="F7" t="n">
+        <v>33</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="I7" t="n">
         <v>120</v>
       </c>
-      <c r="G7" t="n">
+      <c r="J7" t="n">
         <v>0.8113957047462463</v>
       </c>
-      <c r="H7" t="n">
+      <c r="K7" t="n">
         <v>0.1094858050346375</v>
       </c>
-      <c r="I7" t="n">
+      <c r="L7" t="n">
         <v>0.1613653995345229</v>
       </c>
-      <c r="J7" t="n">
+      <c r="M7" t="n">
         <v>14.1155934833204</v>
       </c>
-      <c r="K7" t="n">
+      <c r="N7" t="n">
         <v>21.85499500862441</v>
       </c>
-      <c r="L7" t="n">
+      <c r="O7" t="n">
         <v>0.710596755252824</v>
       </c>
-      <c r="M7" t="n">
+      <c r="P7" t="n">
         <v>0.8113957409221053</v>
       </c>
-      <c r="N7" t="n">
+      <c r="Q7" t="n">
         <v>0.6532195500387897</v>
       </c>
     </row>
@@ -780,34 +849,43 @@
       <c r="D8" t="n">
         <v>150</v>
       </c>
-      <c r="E8" t="b">
-        <v>1</v>
+      <c r="E8" t="n">
+        <v>90</v>
       </c>
       <c r="F8" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>125.5</v>
+      </c>
+      <c r="I8" t="n">
         <v>124</v>
       </c>
-      <c r="G8" t="n">
+      <c r="J8" t="n">
         <v>0.5487590432167053</v>
       </c>
-      <c r="H8" t="n">
+      <c r="K8" t="n">
         <v>0.01905685663223267</v>
       </c>
-      <c r="I8" t="n">
+      <c r="L8" t="n">
         <v>0.2121896162528217</v>
       </c>
-      <c r="J8" t="n">
+      <c r="M8" t="n">
         <v>7.141459744168547</v>
       </c>
-      <c r="K8" t="n">
+      <c r="N8" t="n">
         <v>9.39954211778841</v>
       </c>
-      <c r="L8" t="n">
+      <c r="O8" t="n">
         <v>0.4568966437739098</v>
       </c>
-      <c r="M8" t="n">
+      <c r="P8" t="n">
         <v>0.5487590803472112</v>
       </c>
-      <c r="N8" t="n">
+      <c r="Q8" t="n">
         <v>0.3468773513920241</v>
       </c>
     </row>
@@ -826,34 +904,43 @@
       <c r="D9" t="n">
         <v>136</v>
       </c>
-      <c r="E9" t="b">
-        <v>1</v>
+      <c r="E9" t="n">
+        <v>97</v>
       </c>
       <c r="F9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>125.5</v>
+      </c>
+      <c r="I9" t="n">
         <v>124</v>
       </c>
-      <c r="G9" t="n">
+      <c r="J9" t="n">
         <v>0.547282338142395</v>
       </c>
-      <c r="H9" t="n">
+      <c r="K9" t="n">
         <v>0.2018294930458069</v>
       </c>
-      <c r="I9" t="n">
+      <c r="L9" t="n">
         <v>0.2630937880633374</v>
       </c>
-      <c r="J9" t="n">
+      <c r="M9" t="n">
         <v>7.332521315468941</v>
       </c>
-      <c r="K9" t="n">
+      <c r="N9" t="n">
         <v>10.04193400145842</v>
       </c>
-      <c r="L9" t="n">
+      <c r="O9" t="n">
         <v>0.5762981162770927</v>
       </c>
-      <c r="M9" t="n">
+      <c r="P9" t="n">
         <v>0.5472822837152923</v>
       </c>
-      <c r="N9" t="n">
+      <c r="Q9" t="n">
         <v>0.3970767356881851</v>
       </c>
     </row>
@@ -872,34 +959,43 @@
       <c r="D10" t="n">
         <v>188</v>
       </c>
-      <c r="E10" t="b">
-        <v>1</v>
+      <c r="E10" t="n">
+        <v>88</v>
       </c>
       <c r="F10" t="n">
+        <v>39</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="I10" t="n">
         <v>154</v>
       </c>
-      <c r="G10" t="n">
+      <c r="J10" t="n">
         <v>0.6088144779205322</v>
       </c>
-      <c r="H10" t="n">
+      <c r="K10" t="n">
         <v>0.02627724409103394</v>
       </c>
-      <c r="I10" t="n">
+      <c r="L10" t="n">
         <v>0.2628012048192771</v>
       </c>
-      <c r="J10" t="n">
+      <c r="M10" t="n">
         <v>5.867469879518072</v>
       </c>
-      <c r="K10" t="n">
+      <c r="N10" t="n">
         <v>7.428575565999113</v>
       </c>
-      <c r="L10" t="n">
+      <c r="O10" t="n">
         <v>0.5258659484073805</v>
       </c>
-      <c r="M10" t="n">
+      <c r="P10" t="n">
         <v>0.6088145072029046</v>
       </c>
-      <c r="N10" t="n">
+      <c r="Q10" t="n">
         <v>0.5399096385542169</v>
       </c>
     </row>
@@ -918,34 +1014,43 @@
       <c r="D11" t="n">
         <v>179</v>
       </c>
-      <c r="E11" t="b">
-        <v>1</v>
+      <c r="E11" t="n">
+        <v>102</v>
       </c>
       <c r="F11" t="n">
+        <v>36</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="I11" t="n">
         <v>154</v>
       </c>
-      <c r="G11" t="n">
+      <c r="J11" t="n">
         <v>0.5760010480880737</v>
       </c>
-      <c r="H11" t="n">
+      <c r="K11" t="n">
         <v>0.2133519947528839</v>
       </c>
-      <c r="I11" t="n">
+      <c r="L11" t="n">
         <v>0.2938931297709924</v>
       </c>
-      <c r="J11" t="n">
+      <c r="M11" t="n">
         <v>5.653148854961832</v>
       </c>
-      <c r="K11" t="n">
+      <c r="N11" t="n">
         <v>7.264791439297383</v>
       </c>
-      <c r="L11" t="n">
+      <c r="O11" t="n">
         <v>0.540663246983777</v>
       </c>
-      <c r="M11" t="n">
+      <c r="P11" t="n">
         <v>0.5760010453006176</v>
       </c>
-      <c r="N11" t="n">
+      <c r="Q11" t="n">
         <v>0.5720419847328244</v>
       </c>
     </row>
@@ -964,34 +1069,43 @@
       <c r="D12" t="n">
         <v>157</v>
       </c>
-      <c r="E12" t="b">
-        <v>1</v>
+      <c r="E12" t="n">
+        <v>82</v>
       </c>
       <c r="F12" t="n">
+        <v>38</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>136.5</v>
+      </c>
+      <c r="I12" t="n">
         <v>129</v>
       </c>
-      <c r="G12" t="n">
+      <c r="J12" t="n">
         <v>0.4949547052383423</v>
       </c>
-      <c r="H12" t="n">
+      <c r="K12" t="n">
         <v>0.02863383293151855</v>
       </c>
-      <c r="I12" t="n">
+      <c r="L12" t="n">
         <v>0.2463193657984145</v>
       </c>
-      <c r="J12" t="n">
+      <c r="M12" t="n">
         <v>5.70158550396376</v>
       </c>
-      <c r="K12" t="n">
+      <c r="N12" t="n">
         <v>7.01297131780936</v>
       </c>
-      <c r="L12" t="n">
+      <c r="O12" t="n">
         <v>0.4646132819739173</v>
       </c>
-      <c r="M12" t="n">
+      <c r="P12" t="n">
         <v>0.4949546949864694</v>
       </c>
-      <c r="N12" t="n">
+      <c r="Q12" t="n">
         <v>0.5877689694224235</v>
       </c>
     </row>
@@ -1010,34 +1124,43 @@
       <c r="D13" t="n">
         <v>147</v>
       </c>
-      <c r="E13" t="b">
-        <v>1</v>
+      <c r="E13" t="n">
+        <v>82</v>
       </c>
       <c r="F13" t="n">
+        <v>39</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>136.5</v>
+      </c>
+      <c r="I13" t="n">
         <v>129</v>
       </c>
-      <c r="G13" t="n">
+      <c r="J13" t="n">
         <v>0.4767608046531677</v>
       </c>
-      <c r="H13" t="n">
+      <c r="K13" t="n">
         <v>0.09852075576782227</v>
       </c>
-      <c r="I13" t="n">
+      <c r="L13" t="n">
         <v>0.227112676056338</v>
       </c>
-      <c r="J13" t="n">
+      <c r="M13" t="n">
         <v>5.984154929577465</v>
       </c>
-      <c r="K13" t="n">
+      <c r="N13" t="n">
         <v>7.345154258408207</v>
       </c>
-      <c r="L13" t="n">
+      <c r="O13" t="n">
         <v>0.5273767593446932</v>
       </c>
-      <c r="M13" t="n">
+      <c r="P13" t="n">
         <v>0.4767607928160177</v>
       </c>
-      <c r="N13" t="n">
+      <c r="Q13" t="n">
         <v>0.5557511737089202</v>
       </c>
     </row>
@@ -1056,34 +1179,43 @@
       <c r="D14" t="n">
         <v>151</v>
       </c>
-      <c r="E14" t="b">
-        <v>1</v>
+      <c r="E14" t="n">
+        <v>107</v>
       </c>
       <c r="F14" t="n">
+        <v>35</v>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="I14" t="n">
         <v>136</v>
       </c>
-      <c r="G14" t="n">
+      <c r="J14" t="n">
         <v>0.5613628029823303</v>
       </c>
-      <c r="H14" t="n">
+      <c r="K14" t="n">
         <v>0.03076344728469849</v>
       </c>
-      <c r="I14" t="n">
+      <c r="L14" t="n">
         <v>0.2873453853472883</v>
       </c>
-      <c r="J14" t="n">
+      <c r="M14" t="n">
         <v>6.290675547098002</v>
       </c>
-      <c r="K14" t="n">
+      <c r="N14" t="n">
         <v>8.518882591569382</v>
       </c>
-      <c r="L14" t="n">
+      <c r="O14" t="n">
         <v>0.5455152927506245</v>
       </c>
-      <c r="M14" t="n">
+      <c r="P14" t="n">
         <v>0.5613627583984478</v>
       </c>
-      <c r="N14" t="n">
+      <c r="Q14" t="n">
         <v>0.5761179828734538</v>
       </c>
     </row>
@@ -1102,34 +1234,43 @@
       <c r="D15" t="n">
         <v>150</v>
       </c>
-      <c r="E15" t="b">
-        <v>1</v>
+      <c r="E15" t="n">
+        <v>90</v>
       </c>
       <c r="F15" t="n">
+        <v>34</v>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="I15" t="n">
         <v>136</v>
       </c>
-      <c r="G15" t="n">
+      <c r="J15" t="n">
         <v>0.6389179825782776</v>
       </c>
-      <c r="H15" t="n">
+      <c r="K15" t="n">
         <v>0.03634810447692871</v>
       </c>
-      <c r="I15" t="n">
+      <c r="L15" t="n">
         <v>0.2865384615384615</v>
       </c>
-      <c r="J15" t="n">
+      <c r="M15" t="n">
         <v>5.7125</v>
       </c>
-      <c r="K15" t="n">
+      <c r="N15" t="n">
         <v>7.705829461667816</v>
       </c>
-      <c r="L15" t="n">
+      <c r="O15" t="n">
         <v>0.6614577579813864</v>
       </c>
-      <c r="M15" t="n">
+      <c r="P15" t="n">
         <v>0.6389179826968971</v>
       </c>
-      <c r="N15" t="n">
+      <c r="Q15" t="n">
         <v>0.5201923076923077</v>
       </c>
     </row>
@@ -1148,34 +1289,43 @@
       <c r="D16" t="n">
         <v>141</v>
       </c>
-      <c r="E16" t="b">
-        <v>1</v>
+      <c r="E16" t="n">
+        <v>88</v>
       </c>
       <c r="F16" t="n">
+        <v>34</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="I16" t="n">
         <v>123</v>
       </c>
-      <c r="G16" t="n">
+      <c r="J16" t="n">
         <v>0.5512155294418335</v>
       </c>
-      <c r="H16" t="n">
+      <c r="K16" t="n">
         <v>0.07657504081726074</v>
       </c>
-      <c r="I16" t="n">
+      <c r="L16" t="n">
         <v>0.2466555183946488</v>
       </c>
-      <c r="J16" t="n">
+      <c r="M16" t="n">
         <v>6.137959866220736</v>
       </c>
-      <c r="K16" t="n">
+      <c r="N16" t="n">
         <v>7.78048540756022</v>
       </c>
-      <c r="L16" t="n">
+      <c r="O16" t="n">
         <v>0.6137684884198465</v>
       </c>
-      <c r="M16" t="n">
+      <c r="P16" t="n">
         <v>0.5512155610204151</v>
       </c>
-      <c r="N16" t="n">
+      <c r="Q16" t="n">
         <v>0.5292642140468228</v>
       </c>
     </row>
@@ -1194,34 +1344,43 @@
       <c r="D17" t="n">
         <v>156</v>
       </c>
-      <c r="E17" t="b">
-        <v>1</v>
+      <c r="E17" t="n">
+        <v>97</v>
       </c>
       <c r="F17" t="n">
+        <v>35</v>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="I17" t="n">
         <v>123</v>
       </c>
-      <c r="G17" t="n">
+      <c r="J17" t="n">
         <v>0.4902864992618561</v>
       </c>
-      <c r="H17" t="n">
+      <c r="K17" t="n">
         <v>0.1028748154640198</v>
       </c>
-      <c r="I17" t="n">
+      <c r="L17" t="n">
         <v>0.2854700854700855</v>
       </c>
-      <c r="J17" t="n">
+      <c r="M17" t="n">
         <v>5.662678062678062</v>
       </c>
-      <c r="K17" t="n">
+      <c r="N17" t="n">
         <v>7.320968596885333</v>
       </c>
-      <c r="L17" t="n">
+      <c r="O17" t="n">
         <v>0.5440580120643865</v>
       </c>
-      <c r="M17" t="n">
+      <c r="P17" t="n">
         <v>0.4902864909885646</v>
       </c>
-      <c r="N17" t="n">
+      <c r="Q17" t="n">
         <v>0.5880341880341881</v>
       </c>
     </row>
@@ -1240,34 +1399,43 @@
       <c r="D18" t="n">
         <v>170</v>
       </c>
-      <c r="E18" t="b">
-        <v>1</v>
+      <c r="E18" t="n">
+        <v>106</v>
       </c>
       <c r="F18" t="n">
+        <v>41</v>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" t="n">
+        <v>126</v>
+      </c>
+      <c r="I18" t="n">
         <v>153</v>
       </c>
-      <c r="G18" t="n">
+      <c r="J18" t="n">
         <v>0.4628634452819824</v>
       </c>
-      <c r="H18" t="n">
+      <c r="K18" t="n">
         <v>0.213080108165741</v>
       </c>
-      <c r="I18" t="n">
+      <c r="L18" t="n">
         <v>0.2923005993545413</v>
       </c>
-      <c r="J18" t="n">
+      <c r="M18" t="n">
         <v>5.826187183033656</v>
       </c>
-      <c r="K18" t="n">
+      <c r="N18" t="n">
         <v>7.498854991742609</v>
       </c>
-      <c r="L18" t="n">
+      <c r="O18" t="n">
         <v>0.5675602269453806</v>
       </c>
-      <c r="M18" t="n">
+      <c r="P18" t="n">
         <v>0.4628634240215607</v>
       </c>
-      <c r="N18" t="n">
+      <c r="Q18" t="n">
         <v>0.702166897187644</v>
       </c>
     </row>
@@ -1286,34 +1454,43 @@
       <c r="D19" t="n">
         <v>181</v>
       </c>
-      <c r="E19" t="b">
-        <v>1</v>
+      <c r="E19" t="n">
+        <v>99</v>
       </c>
       <c r="F19" t="n">
+        <v>41</v>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>126</v>
+      </c>
+      <c r="I19" t="n">
         <v>153</v>
       </c>
-      <c r="G19" t="n">
+      <c r="J19" t="n">
         <v>0.4506431221961975</v>
       </c>
-      <c r="H19" t="n">
+      <c r="K19" t="n">
         <v>0.08461993932723999</v>
       </c>
-      <c r="I19" t="n">
+      <c r="L19" t="n">
         <v>0.2999449642267474</v>
       </c>
-      <c r="J19" t="n">
+      <c r="M19" t="n">
         <v>5.632911392405063</v>
       </c>
-      <c r="K19" t="n">
+      <c r="N19" t="n">
         <v>7.269291415846356</v>
       </c>
-      <c r="L19" t="n">
+      <c r="O19" t="n">
         <v>0.5792751913777077</v>
       </c>
-      <c r="M19" t="n">
+      <c r="P19" t="n">
         <v>0.4506431390609977</v>
       </c>
-      <c r="N19" t="n">
+      <c r="Q19" t="n">
         <v>0.7369290038525041</v>
       </c>
     </row>
@@ -1332,34 +1509,43 @@
       <c r="D20" t="n">
         <v>134</v>
       </c>
-      <c r="E20" t="b">
-        <v>1</v>
+      <c r="E20" t="n">
+        <v>97</v>
       </c>
       <c r="F20" t="n">
+        <v>43</v>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>134.5</v>
+      </c>
+      <c r="I20" t="n">
         <v>133</v>
       </c>
-      <c r="G20" t="n">
+      <c r="J20" t="n">
         <v>0.5791653394699097</v>
       </c>
-      <c r="H20" t="n">
+      <c r="K20" t="n">
         <v>0.09511768817901611</v>
       </c>
-      <c r="I20" t="n">
+      <c r="L20" t="n">
         <v>0.2668435013262599</v>
       </c>
-      <c r="J20" t="n">
+      <c r="M20" t="n">
         <v>5.669496021220159</v>
       </c>
-      <c r="K20" t="n">
+      <c r="N20" t="n">
         <v>7.245194144830521</v>
       </c>
-      <c r="L20" t="n">
+      <c r="O20" t="n">
         <v>0.5662435428267696</v>
       </c>
-      <c r="M20" t="n">
+      <c r="P20" t="n">
         <v>0.57916533948396</v>
       </c>
-      <c r="N20" t="n">
+      <c r="Q20" t="n">
         <v>0.5453580901856764</v>
       </c>
     </row>
@@ -1378,34 +1564,43 @@
       <c r="D21" t="n">
         <v>136</v>
       </c>
-      <c r="E21" t="b">
-        <v>1</v>
+      <c r="E21" t="n">
+        <v>106</v>
       </c>
       <c r="F21" t="n">
+        <v>42</v>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>134.5</v>
+      </c>
+      <c r="I21" t="n">
         <v>133</v>
       </c>
-      <c r="G21" t="n">
+      <c r="J21" t="n">
         <v>0.5690152645111084</v>
       </c>
-      <c r="H21" t="n">
+      <c r="K21" t="n">
         <v>0.1273511946201324</v>
       </c>
-      <c r="I21" t="n">
+      <c r="L21" t="n">
         <v>0.2590206185567011</v>
       </c>
-      <c r="J21" t="n">
+      <c r="M21" t="n">
         <v>5.941580756013746</v>
       </c>
-      <c r="K21" t="n">
+      <c r="N21" t="n">
         <v>7.570799846071639</v>
       </c>
-      <c r="L21" t="n">
+      <c r="O21" t="n">
         <v>0.5136536222582581</v>
       </c>
-      <c r="M21" t="n">
+      <c r="P21" t="n">
         <v>0.5690152307591907</v>
       </c>
-      <c r="N21" t="n">
+      <c r="Q21" t="n">
         <v>0.593213058419244</v>
       </c>
     </row>
@@ -1424,34 +1619,43 @@
       <c r="D22" t="n">
         <v>160</v>
       </c>
-      <c r="E22" t="b">
-        <v>1</v>
+      <c r="E22" t="n">
+        <v>95</v>
       </c>
       <c r="F22" t="n">
+        <v>39</v>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>130</v>
+      </c>
+      <c r="I22" t="n">
         <v>134</v>
       </c>
-      <c r="G22" t="n">
+      <c r="J22" t="n">
         <v>0.5919339060783386</v>
       </c>
-      <c r="H22" t="n">
+      <c r="K22" t="n">
         <v>0.08896434307098389</v>
       </c>
-      <c r="I22" t="n">
+      <c r="L22" t="n">
         <v>0.2676232064878353</v>
       </c>
-      <c r="J22" t="n">
+      <c r="M22" t="n">
         <v>5.919525888958203</v>
       </c>
-      <c r="K22" t="n">
+      <c r="N22" t="n">
         <v>7.661954847806894</v>
       </c>
-      <c r="L22" t="n">
+      <c r="O22" t="n">
         <v>0.5431111056974373</v>
       </c>
-      <c r="M22" t="n">
+      <c r="P22" t="n">
         <v>0.5919338358626172</v>
       </c>
-      <c r="N22" t="n">
+      <c r="Q22" t="n">
         <v>0.603243917654398</v>
       </c>
     </row>
@@ -1470,34 +1674,43 @@
       <c r="D23" t="n">
         <v>151</v>
       </c>
-      <c r="E23" t="b">
-        <v>1</v>
+      <c r="E23" t="n">
+        <v>103</v>
       </c>
       <c r="F23" t="n">
+        <v>38</v>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" t="n">
+        <v>130</v>
+      </c>
+      <c r="I23" t="n">
         <v>134</v>
       </c>
-      <c r="G23" t="n">
+      <c r="J23" t="n">
         <v>0.5080452561378479</v>
       </c>
-      <c r="H23" t="n">
+      <c r="K23" t="n">
         <v>0.1358323991298676</v>
       </c>
-      <c r="I23" t="n">
+      <c r="L23" t="n">
         <v>0.2481203007518797</v>
       </c>
-      <c r="J23" t="n">
+      <c r="M23" t="n">
         <v>6.585392051557465</v>
       </c>
-      <c r="K23" t="n">
+      <c r="N23" t="n">
         <v>8.611435456588294</v>
       </c>
-      <c r="L23" t="n">
+      <c r="O23" t="n">
         <v>0.594298698189855</v>
       </c>
-      <c r="M23" t="n">
+      <c r="P23" t="n">
         <v>0.5080452647843285</v>
       </c>
-      <c r="N23" t="n">
+      <c r="Q23" t="n">
         <v>0.6149301825993555</v>
       </c>
     </row>
@@ -1516,34 +1729,43 @@
       <c r="D24" t="n">
         <v>137</v>
       </c>
-      <c r="E24" t="b">
-        <v>1</v>
+      <c r="E24" t="n">
+        <v>102</v>
       </c>
       <c r="F24" t="n">
+        <v>39</v>
+      </c>
+      <c r="G24" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="I24" t="n">
         <v>132</v>
       </c>
-      <c r="G24" t="n">
+      <c r="J24" t="n">
         <v>0.5360705256462097</v>
       </c>
-      <c r="H24" t="n">
+      <c r="K24" t="n">
         <v>0.0709986686706543</v>
       </c>
-      <c r="I24" t="n">
+      <c r="L24" t="n">
         <v>0.2125267665952891</v>
       </c>
-      <c r="J24" t="n">
+      <c r="M24" t="n">
         <v>5.609207708779444</v>
       </c>
-      <c r="K24" t="n">
+      <c r="N24" t="n">
         <v>7.24450615149266</v>
       </c>
-      <c r="L24" t="n">
+      <c r="O24" t="n">
         <v>0.4550775920579175</v>
       </c>
-      <c r="M24" t="n">
+      <c r="P24" t="n">
         <v>0.5360704985925347</v>
       </c>
-      <c r="N24" t="n">
+      <c r="Q24" t="n">
         <v>0.208779443254818</v>
       </c>
     </row>
@@ -1562,34 +1784,43 @@
       <c r="D25" t="n">
         <v>146</v>
       </c>
-      <c r="E25" t="b">
-        <v>1</v>
+      <c r="E25" t="n">
+        <v>105</v>
       </c>
       <c r="F25" t="n">
+        <v>36</v>
+      </c>
+      <c r="G25" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="I25" t="n">
         <v>132</v>
       </c>
-      <c r="G25" t="n">
+      <c r="J25" t="n">
         <v>0.5170442461967468</v>
       </c>
-      <c r="H25" t="n">
+      <c r="K25" t="n">
         <v>0.07097294926643372</v>
       </c>
-      <c r="I25" t="n">
+      <c r="L25" t="n">
         <v>0.2176308539944904</v>
       </c>
-      <c r="J25" t="n">
+      <c r="M25" t="n">
         <v>5.988429752066116</v>
       </c>
-      <c r="K25" t="n">
+      <c r="N25" t="n">
         <v>7.939197314243446</v>
       </c>
-      <c r="L25" t="n">
+      <c r="O25" t="n">
         <v>0.4413872957992682</v>
       </c>
-      <c r="M25" t="n">
+      <c r="P25" t="n">
         <v>0.517044191316135</v>
       </c>
-      <c r="N25" t="n">
+      <c r="Q25" t="n">
         <v>0.2247933884297521</v>
       </c>
     </row>
@@ -1608,34 +1839,43 @@
       <c r="D26" t="n">
         <v>150</v>
       </c>
-      <c r="E26" t="b">
-        <v>1</v>
+      <c r="E26" t="n">
+        <v>96</v>
       </c>
       <c r="F26" t="n">
+        <v>40</v>
+      </c>
+      <c r="G26" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>136</v>
+      </c>
+      <c r="I26" t="n">
         <v>120</v>
       </c>
-      <c r="G26" t="n">
+      <c r="J26" t="n">
         <v>0.5246784687042236</v>
       </c>
-      <c r="H26" t="n">
+      <c r="K26" t="n">
         <v>0.1066404283046722</v>
       </c>
-      <c r="I26" t="n">
+      <c r="L26" t="n">
         <v>0.2698178237321516</v>
       </c>
-      <c r="J26" t="n">
+      <c r="M26" t="n">
         <v>5.804037419990153</v>
       </c>
-      <c r="K26" t="n">
+      <c r="N26" t="n">
         <v>7.695330996982945</v>
       </c>
-      <c r="L26" t="n">
+      <c r="O26" t="n">
         <v>0.5411496017383338</v>
       </c>
-      <c r="M26" t="n">
+      <c r="P26" t="n">
         <v>0.5246783862450679</v>
       </c>
-      <c r="N26" t="n">
+      <c r="Q26" t="n">
         <v>0.638109305760709</v>
       </c>
     </row>
@@ -1654,34 +1894,43 @@
       <c r="D27" t="n">
         <v>145</v>
       </c>
-      <c r="E27" t="b">
-        <v>1</v>
+      <c r="E27" t="n">
+        <v>103</v>
       </c>
       <c r="F27" t="n">
+        <v>38</v>
+      </c>
+      <c r="G27" t="b">
+        <v>1</v>
+      </c>
+      <c r="H27" t="n">
+        <v>136</v>
+      </c>
+      <c r="I27" t="n">
         <v>120</v>
       </c>
-      <c r="G27" t="n">
+      <c r="J27" t="n">
         <v>0.5298634171485901</v>
       </c>
-      <c r="H27" t="n">
+      <c r="K27" t="n">
         <v>0.1783837378025055</v>
       </c>
-      <c r="I27" t="n">
+      <c r="L27" t="n">
         <v>0.2797825012357884</v>
       </c>
-      <c r="J27" t="n">
+      <c r="M27" t="n">
         <v>5.762234305486901</v>
       </c>
-      <c r="K27" t="n">
+      <c r="N27" t="n">
         <v>7.622228595317016</v>
       </c>
-      <c r="L27" t="n">
+      <c r="O27" t="n">
         <v>0.5717760064617589</v>
       </c>
-      <c r="M27" t="n">
+      <c r="P27" t="n">
         <v>0.5298634315334009</v>
       </c>
-      <c r="N27" t="n">
+      <c r="Q27" t="n">
         <v>0.6213544241225902</v>
       </c>
     </row>
@@ -1700,34 +1949,43 @@
       <c r="D28" t="n">
         <v>165</v>
       </c>
-      <c r="E28" t="b">
-        <v>1</v>
+      <c r="E28" t="n">
+        <v>77</v>
       </c>
       <c r="F28" t="n">
+        <v>33</v>
+      </c>
+      <c r="G28" t="b">
+        <v>1</v>
+      </c>
+      <c r="H28" t="n">
+        <v>131</v>
+      </c>
+      <c r="I28" t="n">
         <v>148</v>
       </c>
-      <c r="G28" t="n">
+      <c r="J28" t="n">
         <v>0.6210268139839172</v>
       </c>
-      <c r="H28" t="n">
+      <c r="K28" t="n">
         <v>0.06041842699050903</v>
       </c>
-      <c r="I28" t="n">
+      <c r="L28" t="n">
         <v>0.2229965156794425</v>
       </c>
-      <c r="J28" t="n">
+      <c r="M28" t="n">
         <v>6.945644599303136</v>
       </c>
-      <c r="K28" t="n">
+      <c r="N28" t="n">
         <v>9.109362645370863</v>
       </c>
-      <c r="L28" t="n">
+      <c r="O28" t="n">
         <v>0.5436194280411497</v>
       </c>
-      <c r="M28" t="n">
+      <c r="P28" t="n">
         <v>0.6210268847384389</v>
       </c>
-      <c r="N28" t="n">
+      <c r="Q28" t="n">
         <v>0.5184668989547039</v>
       </c>
     </row>
@@ -1746,34 +2004,43 @@
       <c r="D29" t="n">
         <v>162</v>
       </c>
-      <c r="E29" t="b">
-        <v>1</v>
+      <c r="E29" t="n">
+        <v>79</v>
       </c>
       <c r="F29" t="n">
+        <v>35</v>
+      </c>
+      <c r="G29" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" t="n">
+        <v>131</v>
+      </c>
+      <c r="I29" t="n">
         <v>148</v>
       </c>
-      <c r="G29" t="n">
+      <c r="J29" t="n">
         <v>0.6621218323707581</v>
       </c>
-      <c r="H29" t="n">
+      <c r="K29" t="n">
         <v>0.0485149621963501</v>
       </c>
-      <c r="I29" t="n">
+      <c r="L29" t="n">
         <v>0.2477183833116036</v>
       </c>
-      <c r="J29" t="n">
+      <c r="M29" t="n">
         <v>6.445893089960887</v>
       </c>
-      <c r="K29" t="n">
+      <c r="N29" t="n">
         <v>8.33162085837867</v>
       </c>
-      <c r="L29" t="n">
+      <c r="O29" t="n">
         <v>0.5297270835968723</v>
       </c>
-      <c r="M29" t="n">
+      <c r="P29" t="n">
         <v>0.6621217504590625</v>
       </c>
-      <c r="N29" t="n">
+      <c r="Q29" t="n">
         <v>0.5723598435462842</v>
       </c>
     </row>
@@ -1792,34 +2059,43 @@
       <c r="D30" t="n">
         <v>176</v>
       </c>
-      <c r="E30" t="b">
-        <v>1</v>
+      <c r="E30" t="n">
+        <v>109</v>
       </c>
       <c r="F30" t="n">
+        <v>45</v>
+      </c>
+      <c r="G30" t="b">
+        <v>1</v>
+      </c>
+      <c r="H30" t="n">
+        <v>117</v>
+      </c>
+      <c r="I30" t="n">
         <v>171</v>
       </c>
-      <c r="G30" t="n">
+      <c r="J30" t="n">
         <v>0.4871482849121094</v>
       </c>
-      <c r="H30" t="n">
+      <c r="K30" t="n">
         <v>0.1610651910305023</v>
       </c>
-      <c r="I30" t="n">
+      <c r="L30" t="n">
         <v>0.2788935202728306</v>
       </c>
-      <c r="J30" t="n">
+      <c r="M30" t="n">
         <v>6.374384236453202</v>
       </c>
-      <c r="K30" t="n">
+      <c r="N30" t="n">
         <v>8.867685544250483</v>
       </c>
-      <c r="L30" t="n">
+      <c r="O30" t="n">
         <v>0.5868869461276225</v>
       </c>
-      <c r="M30" t="n">
+      <c r="P30" t="n">
         <v>0.4871482810803924</v>
       </c>
-      <c r="N30" t="n">
+      <c r="Q30" t="n">
         <v>0.5183781735505874</v>
       </c>
     </row>
@@ -1838,34 +2114,43 @@
       <c r="D31" t="n">
         <v>189</v>
       </c>
-      <c r="E31" t="b">
-        <v>1</v>
+      <c r="E31" t="n">
+        <v>94</v>
       </c>
       <c r="F31" t="n">
+        <v>61</v>
+      </c>
+      <c r="G31" t="b">
+        <v>1</v>
+      </c>
+      <c r="H31" t="n">
+        <v>117</v>
+      </c>
+      <c r="I31" t="n">
         <v>171</v>
       </c>
-      <c r="G31" t="n">
+      <c r="J31" t="n">
         <v>0.4243854284286499</v>
       </c>
-      <c r="H31" t="n">
+      <c r="K31" t="n">
         <v>0.05755844712257385</v>
       </c>
-      <c r="I31" t="n">
+      <c r="L31" t="n">
         <v>0.145114479200258</v>
       </c>
-      <c r="J31" t="n">
+      <c r="M31" t="n">
         <v>11.88552079974202</v>
       </c>
-      <c r="K31" t="n">
+      <c r="N31" t="n">
         <v>15.17063007158187</v>
       </c>
-      <c r="L31" t="n">
+      <c r="O31" t="n">
         <v>0.4668729630083333</v>
       </c>
-      <c r="M31" t="n">
+      <c r="P31" t="n">
         <v>0.4243853796871154</v>
       </c>
-      <c r="N31" t="n">
+      <c r="Q31" t="n">
         <v>0.3718155433731055</v>
       </c>
     </row>
@@ -1884,34 +2169,43 @@
       <c r="D32" t="n">
         <v>83</v>
       </c>
-      <c r="E32" t="b">
-        <v>1</v>
+      <c r="E32" t="n">
+        <v>73</v>
       </c>
       <c r="F32" t="n">
+        <v>35</v>
+      </c>
+      <c r="G32" t="b">
+        <v>1</v>
+      </c>
+      <c r="H32" t="n">
+        <v>132</v>
+      </c>
+      <c r="I32" t="n">
         <v>116</v>
       </c>
-      <c r="G32" t="n">
+      <c r="J32" t="n">
         <v>0.715678334236145</v>
       </c>
-      <c r="H32" t="n">
+      <c r="K32" t="n">
         <v>0.0100400447845459</v>
       </c>
-      <c r="I32" t="n">
+      <c r="L32" t="n">
         <v>0.1690721649484536</v>
       </c>
-      <c r="J32" t="n">
+      <c r="M32" t="n">
         <v>7.721649484536083</v>
       </c>
-      <c r="K32" t="n">
+      <c r="N32" t="n">
         <v>10.22307880269861</v>
       </c>
-      <c r="L32" t="n">
+      <c r="O32" t="n">
         <v>0.5541156479138727</v>
       </c>
-      <c r="M32" t="n">
+      <c r="P32" t="n">
         <v>0.7156782756933278</v>
       </c>
-      <c r="N32" t="n">
+      <c r="Q32" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1930,34 +2224,43 @@
       <c r="D33" t="n">
         <v>130</v>
       </c>
-      <c r="E33" t="b">
-        <v>1</v>
+      <c r="E33" t="n">
+        <v>98</v>
       </c>
       <c r="F33" t="n">
+        <v>37</v>
+      </c>
+      <c r="G33" t="b">
+        <v>1</v>
+      </c>
+      <c r="H33" t="n">
+        <v>132</v>
+      </c>
+      <c r="I33" t="n">
         <v>116</v>
       </c>
-      <c r="G33" t="n">
+      <c r="J33" t="n">
         <v>0.6116756796836853</v>
       </c>
-      <c r="H33" t="n">
+      <c r="K33" t="n">
         <v>0.02819520235061646</v>
       </c>
-      <c r="I33" t="n">
+      <c r="L33" t="n">
         <v>0.2051898125901009</v>
       </c>
-      <c r="J33" t="n">
+      <c r="M33" t="n">
         <v>8.018260451705912</v>
       </c>
-      <c r="K33" t="n">
+      <c r="N33" t="n">
         <v>10.30206913896278</v>
       </c>
-      <c r="L33" t="n">
+      <c r="O33" t="n">
         <v>0.5770414033415048</v>
       </c>
-      <c r="M33" t="n">
+      <c r="P33" t="n">
         <v>0.611675710965555</v>
       </c>
-      <c r="N33" t="n">
+      <c r="Q33" t="n">
         <v>0.6756367131186929</v>
       </c>
     </row>
@@ -1976,34 +2279,43 @@
       <c r="D34" t="n">
         <v>70</v>
       </c>
-      <c r="E34" t="b">
-        <v>1</v>
+      <c r="E34" t="n">
+        <v>75</v>
       </c>
       <c r="F34" t="n">
+        <v>30</v>
+      </c>
+      <c r="G34" t="b">
+        <v>1</v>
+      </c>
+      <c r="H34" t="n">
+        <v>129.5</v>
+      </c>
+      <c r="I34" t="n">
         <v>97</v>
       </c>
-      <c r="G34" t="n">
+      <c r="J34" t="n">
         <v>0.5585066080093384</v>
       </c>
-      <c r="H34" t="n">
+      <c r="K34" t="n">
         <v>0.04973524808883667</v>
       </c>
-      <c r="I34" t="n">
+      <c r="L34" t="n">
         <v>0.06040268456375839</v>
       </c>
-      <c r="J34" t="n">
+      <c r="M34" t="n">
         <v>12.43120805369128</v>
       </c>
-      <c r="K34" t="n">
+      <c r="N34" t="n">
         <v>14.5353653424186</v>
       </c>
-      <c r="L34" t="n">
+      <c r="O34" t="n">
         <v>0.5801502514183068</v>
       </c>
-      <c r="M34" t="n">
+      <c r="P34" t="n">
         <v>0.5585066168413028</v>
       </c>
-      <c r="N34" t="n">
+      <c r="Q34" t="n">
         <v>0.2919463087248322</v>
       </c>
     </row>
@@ -2022,34 +2334,43 @@
       <c r="D35" t="n">
         <v>104</v>
       </c>
-      <c r="E35" t="b">
-        <v>1</v>
+      <c r="E35" t="n">
+        <v>91</v>
       </c>
       <c r="F35" t="n">
+        <v>31</v>
+      </c>
+      <c r="G35" t="b">
+        <v>1</v>
+      </c>
+      <c r="H35" t="n">
+        <v>129.5</v>
+      </c>
+      <c r="I35" t="n">
         <v>97</v>
       </c>
-      <c r="G35" t="n">
+      <c r="J35" t="n">
         <v>0.5372719764709473</v>
       </c>
-      <c r="H35" t="n">
+      <c r="K35" t="n">
         <v>0.05613094568252563</v>
       </c>
-      <c r="I35" t="n">
+      <c r="L35" t="n">
         <v>0.1085353003161222</v>
       </c>
-      <c r="J35" t="n">
+      <c r="M35" t="n">
         <v>10.52687038988409</v>
       </c>
-      <c r="K35" t="n">
+      <c r="N35" t="n">
         <v>12.4869584232453</v>
       </c>
-      <c r="L35" t="n">
+      <c r="O35" t="n">
         <v>0.5382238987438723</v>
       </c>
-      <c r="M35" t="n">
+      <c r="P35" t="n">
         <v>0.5372719869658457</v>
       </c>
-      <c r="N35" t="n">
+      <c r="Q35" t="n">
         <v>0.4478398314014753</v>
       </c>
     </row>
@@ -2068,34 +2389,43 @@
       <c r="D36" t="n">
         <v>139</v>
       </c>
-      <c r="E36" t="b">
-        <v>1</v>
+      <c r="E36" t="n">
+        <v>105</v>
       </c>
       <c r="F36" t="n">
+        <v>39</v>
+      </c>
+      <c r="G36" t="b">
+        <v>1</v>
+      </c>
+      <c r="H36" t="n">
+        <v>128</v>
+      </c>
+      <c r="I36" t="n">
         <v>130</v>
       </c>
-      <c r="G36" t="n">
+      <c r="J36" t="n">
         <v>0.6718750596046448</v>
       </c>
-      <c r="H36" t="n">
+      <c r="K36" t="n">
         <v>0.214832991361618</v>
       </c>
-      <c r="I36" t="n">
+      <c r="L36" t="n">
         <v>0.3081800887761573</v>
       </c>
-      <c r="J36" t="n">
+      <c r="M36" t="n">
         <v>5.14140773620799</v>
       </c>
-      <c r="K36" t="n">
+      <c r="N36" t="n">
         <v>6.900047328741396</v>
       </c>
-      <c r="L36" t="n">
+      <c r="O36" t="n">
         <v>0.6516501826996167</v>
       </c>
-      <c r="M36" t="n">
+      <c r="P36" t="n">
         <v>0.6718750402468018</v>
       </c>
-      <c r="N36" t="n">
+      <c r="Q36" t="n">
         <v>0.6766011414077362</v>
       </c>
     </row>
@@ -2114,34 +2444,43 @@
       <c r="D37" t="n">
         <v>177</v>
       </c>
-      <c r="E37" t="b">
-        <v>1</v>
+      <c r="E37" t="n">
+        <v>100</v>
       </c>
       <c r="F37" t="n">
+        <v>43</v>
+      </c>
+      <c r="G37" t="b">
+        <v>1</v>
+      </c>
+      <c r="H37" t="n">
+        <v>128</v>
+      </c>
+      <c r="I37" t="n">
         <v>130</v>
       </c>
-      <c r="G37" t="n">
+      <c r="J37" t="n">
         <v>0.4974704384803772</v>
       </c>
-      <c r="H37" t="n">
+      <c r="K37" t="n">
         <v>0.1230161488056183</v>
       </c>
-      <c r="I37" t="n">
+      <c r="L37" t="n">
         <v>0.2891335567257061</v>
       </c>
-      <c r="J37" t="n">
+      <c r="M37" t="n">
         <v>5.261369076112973</v>
       </c>
-      <c r="K37" t="n">
+      <c r="N37" t="n">
         <v>6.799283323256139</v>
       </c>
-      <c r="L37" t="n">
+      <c r="O37" t="n">
         <v>0.5132253772945929</v>
       </c>
-      <c r="M37" t="n">
+      <c r="P37" t="n">
         <v>0.4974704756067978</v>
       </c>
-      <c r="N37" t="n">
+      <c r="Q37" t="n">
         <v>0.700813786500718</v>
       </c>
     </row>
@@ -2160,34 +2499,43 @@
       <c r="D38" t="n">
         <v>129</v>
       </c>
-      <c r="E38" t="b">
-        <v>1</v>
+      <c r="E38" t="n">
+        <v>99</v>
       </c>
       <c r="F38" t="n">
+        <v>33</v>
+      </c>
+      <c r="G38" t="b">
+        <v>1</v>
+      </c>
+      <c r="H38" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="I38" t="n">
         <v>129</v>
       </c>
-      <c r="G38" t="n">
+      <c r="J38" t="n">
         <v>0.5800935626029968</v>
       </c>
-      <c r="H38" t="n">
+      <c r="K38" t="n">
         <v>0.1979728937149048</v>
       </c>
-      <c r="I38" t="n">
+      <c r="L38" t="n">
         <v>0.2509673852957435</v>
       </c>
-      <c r="J38" t="n">
+      <c r="M38" t="n">
         <v>7.570480928689884</v>
       </c>
-      <c r="K38" t="n">
+      <c r="N38" t="n">
         <v>10.24964775783816</v>
       </c>
-      <c r="L38" t="n">
+      <c r="O38" t="n">
         <v>0.5394531254861057</v>
       </c>
-      <c r="M38" t="n">
+      <c r="P38" t="n">
         <v>0.5800935178622035</v>
       </c>
-      <c r="N38" t="n">
+      <c r="Q38" t="n">
         <v>0.761746821448314</v>
       </c>
     </row>
@@ -2206,34 +2554,43 @@
       <c r="D39" t="n">
         <v>146</v>
       </c>
-      <c r="E39" t="b">
-        <v>1</v>
+      <c r="E39" t="n">
+        <v>87</v>
       </c>
       <c r="F39" t="n">
+        <v>34</v>
+      </c>
+      <c r="G39" t="b">
+        <v>1</v>
+      </c>
+      <c r="H39" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="I39" t="n">
         <v>129</v>
       </c>
-      <c r="G39" t="n">
+      <c r="J39" t="n">
         <v>0.652454674243927</v>
       </c>
-      <c r="H39" t="n">
+      <c r="K39" t="n">
         <v>0.1314727663993835</v>
       </c>
-      <c r="I39" t="n">
+      <c r="L39" t="n">
         <v>0.2274220032840722</v>
       </c>
-      <c r="J39" t="n">
+      <c r="M39" t="n">
         <v>8.608374384236454</v>
       </c>
-      <c r="K39" t="n">
+      <c r="N39" t="n">
         <v>11.81379200108889</v>
       </c>
-      <c r="L39" t="n">
+      <c r="O39" t="n">
         <v>0.5908148004852581</v>
       </c>
-      <c r="M39" t="n">
+      <c r="P39" t="n">
         <v>0.6524546321950813</v>
       </c>
-      <c r="N39" t="n">
+      <c r="Q39" t="n">
         <v>0.6428571428571429</v>
       </c>
     </row>
@@ -2252,34 +2609,43 @@
       <c r="D40" t="n">
         <v>130</v>
       </c>
-      <c r="E40" t="b">
-        <v>1</v>
+      <c r="E40" t="n">
+        <v>84</v>
       </c>
       <c r="F40" t="n">
+        <v>33</v>
+      </c>
+      <c r="G40" t="b">
+        <v>1</v>
+      </c>
+      <c r="H40" t="n">
+        <v>128.5</v>
+      </c>
+      <c r="I40" t="n">
         <v>106</v>
       </c>
-      <c r="G40" t="n">
+      <c r="J40" t="n">
         <v>0.5983039140701294</v>
       </c>
-      <c r="H40" t="n">
+      <c r="K40" t="n">
         <v>0.2119756937026978</v>
       </c>
-      <c r="I40" t="n">
+      <c r="L40" t="n">
         <v>0.237565445026178</v>
       </c>
-      <c r="J40" t="n">
+      <c r="M40" t="n">
         <v>6.289267015706806</v>
       </c>
-      <c r="K40" t="n">
+      <c r="N40" t="n">
         <v>8.104277843936975</v>
       </c>
-      <c r="L40" t="n">
+      <c r="O40" t="n">
         <v>0.5655503399270646</v>
       </c>
-      <c r="M40" t="n">
+      <c r="P40" t="n">
         <v>0.5983038366020121</v>
       </c>
-      <c r="N40" t="n">
+      <c r="Q40" t="n">
         <v>0.6007853403141361</v>
       </c>
     </row>
@@ -2298,34 +2664,43 @@
       <c r="D41" t="n">
         <v>134</v>
       </c>
-      <c r="E41" t="b">
-        <v>1</v>
+      <c r="E41" t="n">
+        <v>85</v>
       </c>
       <c r="F41" t="n">
+        <v>33</v>
+      </c>
+      <c r="G41" t="b">
+        <v>1</v>
+      </c>
+      <c r="H41" t="n">
+        <v>128.5</v>
+      </c>
+      <c r="I41" t="n">
         <v>106</v>
       </c>
-      <c r="G41" t="n">
+      <c r="J41" t="n">
         <v>0.5984174013137817</v>
       </c>
-      <c r="H41" t="n">
+      <c r="K41" t="n">
         <v>0.1590598821640015</v>
       </c>
-      <c r="I41" t="n">
+      <c r="L41" t="n">
         <v>0.2284299858557284</v>
       </c>
-      <c r="J41" t="n">
+      <c r="M41" t="n">
         <v>7.054455445544554</v>
       </c>
-      <c r="K41" t="n">
+      <c r="N41" t="n">
         <v>9.276401597129706</v>
       </c>
-      <c r="L41" t="n">
+      <c r="O41" t="n">
         <v>0.6001101738875444</v>
       </c>
-      <c r="M41" t="n">
+      <c r="P41" t="n">
         <v>0.5984173944416054</v>
       </c>
-      <c r="N41" t="n">
+      <c r="Q41" t="n">
         <v>0.5721357850070722</v>
       </c>
     </row>
@@ -2344,34 +2719,43 @@
       <c r="D42" t="n">
         <v>175</v>
       </c>
-      <c r="E42" t="b">
-        <v>1</v>
+      <c r="E42" t="n">
+        <v>90</v>
       </c>
       <c r="F42" t="n">
+        <v>40</v>
+      </c>
+      <c r="G42" t="b">
+        <v>1</v>
+      </c>
+      <c r="H42" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="I42" t="n">
         <v>163</v>
       </c>
-      <c r="G42" t="n">
+      <c r="J42" t="n">
         <v>0.6176156997680664</v>
       </c>
-      <c r="H42" t="n">
+      <c r="K42" t="n">
         <v>0.1887101233005524</v>
       </c>
-      <c r="I42" t="n">
+      <c r="L42" t="n">
         <v>0.2818352059925094</v>
       </c>
-      <c r="J42" t="n">
+      <c r="M42" t="n">
         <v>5.74063670411985</v>
       </c>
-      <c r="K42" t="n">
+      <c r="N42" t="n">
         <v>7.35222710786962</v>
       </c>
-      <c r="L42" t="n">
+      <c r="O42" t="n">
         <v>0.532274876860428</v>
       </c>
-      <c r="M42" t="n">
+      <c r="P42" t="n">
         <v>0.6176156289564775</v>
       </c>
-      <c r="N42" t="n">
+      <c r="Q42" t="n">
         <v>0.4480337078651686</v>
       </c>
     </row>
@@ -2390,34 +2774,43 @@
       <c r="D43" t="n">
         <v>174</v>
       </c>
-      <c r="E43" t="b">
-        <v>1</v>
+      <c r="E43" t="n">
+        <v>92</v>
       </c>
       <c r="F43" t="n">
+        <v>41</v>
+      </c>
+      <c r="G43" t="b">
+        <v>1</v>
+      </c>
+      <c r="H43" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="I43" t="n">
         <v>163</v>
       </c>
-      <c r="G43" t="n">
+      <c r="J43" t="n">
         <v>0.5875904560089111</v>
       </c>
-      <c r="H43" t="n">
+      <c r="K43" t="n">
         <v>0.1173776984214783</v>
       </c>
-      <c r="I43" t="n">
+      <c r="L43" t="n">
         <v>0.2620967741935484</v>
       </c>
-      <c r="J43" t="n">
+      <c r="M43" t="n">
         <v>6.087701612903226</v>
       </c>
-      <c r="K43" t="n">
+      <c r="N43" t="n">
         <v>8.167228969011342</v>
       </c>
-      <c r="L43" t="n">
+      <c r="O43" t="n">
         <v>0.5295296094162512</v>
       </c>
-      <c r="M43" t="n">
+      <c r="P43" t="n">
         <v>0.5875905326930061</v>
       </c>
-      <c r="N43" t="n">
+      <c r="Q43" t="n">
         <v>0.4445564516129032</v>
       </c>
     </row>
@@ -2436,34 +2829,43 @@
       <c r="D44" t="n">
         <v>179</v>
       </c>
-      <c r="E44" t="b">
-        <v>1</v>
+      <c r="E44" t="n">
+        <v>88</v>
       </c>
       <c r="F44" t="n">
+        <v>33</v>
+      </c>
+      <c r="G44" t="b">
+        <v>1</v>
+      </c>
+      <c r="H44" t="n">
+        <v>126</v>
+      </c>
+      <c r="I44" t="n">
         <v>171</v>
       </c>
-      <c r="G44" t="n">
+      <c r="J44" t="n">
         <v>0.5038752555847168</v>
       </c>
-      <c r="H44" t="n">
+      <c r="K44" t="n">
         <v>0.04617679119110107</v>
       </c>
-      <c r="I44" t="n">
+      <c r="L44" t="n">
         <v>0.268259385665529</v>
       </c>
-      <c r="J44" t="n">
+      <c r="M44" t="n">
         <v>6.292150170648465</v>
       </c>
-      <c r="K44" t="n">
+      <c r="N44" t="n">
         <v>8.230219849513807</v>
       </c>
-      <c r="L44" t="n">
+      <c r="O44" t="n">
         <v>0.5235129259585456</v>
       </c>
-      <c r="M44" t="n">
+      <c r="P44" t="n">
         <v>0.5038752647702459</v>
       </c>
-      <c r="N44" t="n">
+      <c r="Q44" t="n">
         <v>0.4921501706484642</v>
       </c>
     </row>
@@ -2482,34 +2884,43 @@
       <c r="D45" t="n">
         <v>185</v>
       </c>
-      <c r="E45" t="b">
-        <v>1</v>
+      <c r="E45" t="n">
+        <v>95</v>
       </c>
       <c r="F45" t="n">
+        <v>43</v>
+      </c>
+      <c r="G45" t="b">
+        <v>1</v>
+      </c>
+      <c r="H45" t="n">
+        <v>126</v>
+      </c>
+      <c r="I45" t="n">
         <v>171</v>
       </c>
-      <c r="G45" t="n">
+      <c r="J45" t="n">
         <v>0.4627314507961273</v>
       </c>
-      <c r="H45" t="n">
+      <c r="K45" t="n">
         <v>0.06761622428894043</v>
       </c>
-      <c r="I45" t="n">
+      <c r="L45" t="n">
         <v>0.337468982630273</v>
       </c>
-      <c r="J45" t="n">
+      <c r="M45" t="n">
         <v>5.046650124069479</v>
       </c>
-      <c r="K45" t="n">
+      <c r="N45" t="n">
         <v>6.566891919234562</v>
       </c>
-      <c r="L45" t="n">
+      <c r="O45" t="n">
         <v>0.5521420754222816</v>
       </c>
-      <c r="M45" t="n">
+      <c r="P45" t="n">
         <v>0.4627314286103085</v>
       </c>
-      <c r="N45" t="n">
+      <c r="Q45" t="n">
         <v>0.5617866004962779</v>
       </c>
     </row>
@@ -2528,34 +2939,43 @@
       <c r="D46" t="n">
         <v>228</v>
       </c>
-      <c r="E46" t="b">
-        <v>1</v>
+      <c r="E46" t="n">
+        <v>71</v>
       </c>
       <c r="F46" t="n">
+        <v>30</v>
+      </c>
+      <c r="G46" t="b">
+        <v>1</v>
+      </c>
+      <c r="H46" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="I46" t="n">
         <v>120</v>
       </c>
-      <c r="G46" t="n">
+      <c r="J46" t="n">
         <v>0.8687027096748352</v>
       </c>
-      <c r="H46" t="n">
+      <c r="K46" t="n">
         <v>0.003988385200500488</v>
       </c>
-      <c r="I46" t="n">
+      <c r="L46" t="n">
         <v>0.04899497487437186</v>
       </c>
-      <c r="J46" t="n">
+      <c r="M46" t="n">
         <v>25.26884422110553</v>
       </c>
-      <c r="K46" t="n">
+      <c r="N46" t="n">
         <v>36.55040575430073</v>
       </c>
-      <c r="L46" t="n">
+      <c r="O46" t="n">
         <v>0.6575366295629865</v>
       </c>
-      <c r="M46" t="n">
+      <c r="P46" t="n">
         <v>0.8687027800523475</v>
       </c>
-      <c r="N46" t="n">
+      <c r="Q46" t="n">
         <v>0.5778894472361809</v>
       </c>
     </row>
@@ -2574,34 +2994,43 @@
       <c r="D47" t="n">
         <v>111</v>
       </c>
-      <c r="E47" t="b">
-        <v>1</v>
+      <c r="E47" t="n">
+        <v>86</v>
       </c>
       <c r="F47" t="n">
+        <v>33</v>
+      </c>
+      <c r="G47" t="b">
+        <v>1</v>
+      </c>
+      <c r="H47" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="I47" t="n">
         <v>120</v>
       </c>
-      <c r="G47" t="n">
+      <c r="J47" t="n">
         <v>0.8736600279808044</v>
       </c>
-      <c r="H47" t="n">
+      <c r="K47" t="n">
         <v>0.03023731708526611</v>
       </c>
-      <c r="I47" t="n">
+      <c r="L47" t="n">
         <v>0.1541666666666667</v>
       </c>
-      <c r="J47" t="n">
+      <c r="M47" t="n">
         <v>13.47333333333333</v>
       </c>
-      <c r="K47" t="n">
+      <c r="N47" t="n">
         <v>19.63071572816437</v>
       </c>
-      <c r="L47" t="n">
+      <c r="O47" t="n">
         <v>0.750230124727046</v>
       </c>
-      <c r="M47" t="n">
+      <c r="P47" t="n">
         <v>0.8736599703497775</v>
       </c>
-      <c r="N47" t="n">
+      <c r="Q47" t="n">
         <v>0.7225</v>
       </c>
     </row>
@@ -2620,34 +3049,43 @@
       <c r="D48" t="n">
         <v>146</v>
       </c>
-      <c r="E48" t="b">
-        <v>1</v>
+      <c r="E48" t="n">
+        <v>90</v>
       </c>
       <c r="F48" t="n">
+        <v>30</v>
+      </c>
+      <c r="G48" t="b">
+        <v>1</v>
+      </c>
+      <c r="H48" t="n">
+        <v>129.5</v>
+      </c>
+      <c r="I48" t="n">
         <v>124</v>
       </c>
-      <c r="G48" t="n">
+      <c r="J48" t="n">
         <v>0.5970541834831238</v>
       </c>
-      <c r="H48" t="n">
+      <c r="K48" t="n">
         <v>0.03560948371887207</v>
       </c>
-      <c r="I48" t="n">
+      <c r="L48" t="n">
         <v>0.205030487804878</v>
       </c>
-      <c r="J48" t="n">
+      <c r="M48" t="n">
         <v>8.022103658536585</v>
       </c>
-      <c r="K48" t="n">
+      <c r="N48" t="n">
         <v>10.76802940732765</v>
       </c>
-      <c r="L48" t="n">
+      <c r="O48" t="n">
         <v>0.5326430315285354</v>
       </c>
-      <c r="M48" t="n">
+      <c r="P48" t="n">
         <v>0.5970542427185114</v>
       </c>
-      <c r="N48" t="n">
+      <c r="Q48" t="n">
         <v>0.4047256097560976</v>
       </c>
     </row>
@@ -2666,34 +3104,43 @@
       <c r="D49" t="n">
         <v>133</v>
       </c>
-      <c r="E49" t="b">
-        <v>1</v>
+      <c r="E49" t="n">
+        <v>97</v>
       </c>
       <c r="F49" t="n">
+        <v>35</v>
+      </c>
+      <c r="G49" t="b">
+        <v>1</v>
+      </c>
+      <c r="H49" t="n">
+        <v>129.5</v>
+      </c>
+      <c r="I49" t="n">
         <v>124</v>
       </c>
-      <c r="G49" t="n">
+      <c r="J49" t="n">
         <v>0.5148859620094299</v>
       </c>
-      <c r="H49" t="n">
+      <c r="K49" t="n">
         <v>0.04327309131622314</v>
       </c>
-      <c r="I49" t="n">
+      <c r="L49" t="n">
         <v>0.2577447335811648</v>
       </c>
-      <c r="J49" t="n">
+      <c r="M49" t="n">
         <v>7.157992565055762</v>
       </c>
-      <c r="K49" t="n">
+      <c r="N49" t="n">
         <v>9.531302372029922</v>
       </c>
-      <c r="L49" t="n">
+      <c r="O49" t="n">
         <v>0.5685650862861711</v>
       </c>
-      <c r="M49" t="n">
+      <c r="P49" t="n">
         <v>0.5148859986380647</v>
       </c>
-      <c r="N49" t="n">
+      <c r="Q49" t="n">
         <v>0.4535315985130112</v>
       </c>
     </row>
@@ -2712,34 +3159,43 @@
       <c r="D50" t="n">
         <v>185</v>
       </c>
-      <c r="E50" t="b">
-        <v>1</v>
+      <c r="E50" t="n">
+        <v>88</v>
       </c>
       <c r="F50" t="n">
+        <v>39</v>
+      </c>
+      <c r="G50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H50" t="n">
+        <v>128.5</v>
+      </c>
+      <c r="I50" t="n">
         <v>154</v>
       </c>
-      <c r="G50" t="n">
+      <c r="J50" t="n">
         <v>0.6211174130439758</v>
       </c>
-      <c r="H50" t="n">
+      <c r="K50" t="n">
         <v>0.1500807702541351</v>
       </c>
-      <c r="I50" t="n">
+      <c r="L50" t="n">
         <v>0.2861952861952862</v>
       </c>
-      <c r="J50" t="n">
+      <c r="M50" t="n">
         <v>5.678114478114479</v>
       </c>
-      <c r="K50" t="n">
+      <c r="N50" t="n">
         <v>7.227519424881335</v>
       </c>
-      <c r="L50" t="n">
+      <c r="O50" t="n">
         <v>0.5787360470878872</v>
       </c>
-      <c r="M50" t="n">
+      <c r="P50" t="n">
         <v>0.6211173859099201</v>
       </c>
-      <c r="N50" t="n">
+      <c r="Q50" t="n">
         <v>0.5824915824915825</v>
       </c>
     </row>
@@ -2758,34 +3214,43 @@
       <c r="D51" t="n">
         <v>175</v>
       </c>
-      <c r="E51" t="b">
-        <v>1</v>
+      <c r="E51" t="n">
+        <v>102</v>
       </c>
       <c r="F51" t="n">
+        <v>36</v>
+      </c>
+      <c r="G51" t="b">
+        <v>1</v>
+      </c>
+      <c r="H51" t="n">
+        <v>128.5</v>
+      </c>
+      <c r="I51" t="n">
         <v>154</v>
       </c>
-      <c r="G51" t="n">
+      <c r="J51" t="n">
         <v>0.5489990711212158</v>
       </c>
-      <c r="H51" t="n">
+      <c r="K51" t="n">
         <v>0.1215128600597382</v>
       </c>
-      <c r="I51" t="n">
+      <c r="L51" t="n">
         <v>0.2805181863477827</v>
       </c>
-      <c r="J51" t="n">
+      <c r="M51" t="n">
         <v>5.808669656203288</v>
       </c>
-      <c r="K51" t="n">
+      <c r="N51" t="n">
         <v>7.415761772781857</v>
       </c>
-      <c r="L51" t="n">
+      <c r="O51" t="n">
         <v>0.5295035971822016</v>
       </c>
-      <c r="M51" t="n">
+      <c r="P51" t="n">
         <v>0.5489990632635613</v>
       </c>
-      <c r="N51" t="n">
+      <c r="Q51" t="n">
         <v>0.6103637269556552</v>
       </c>
     </row>
@@ -2804,34 +3269,43 @@
       <c r="D52" t="n">
         <v>158</v>
       </c>
-      <c r="E52" t="b">
-        <v>1</v>
+      <c r="E52" t="n">
+        <v>82</v>
       </c>
       <c r="F52" t="n">
+        <v>38</v>
+      </c>
+      <c r="G52" t="b">
+        <v>1</v>
+      </c>
+      <c r="H52" t="n">
+        <v>118.5</v>
+      </c>
+      <c r="I52" t="n">
         <v>129</v>
       </c>
-      <c r="G52" t="n">
+      <c r="J52" t="n">
         <v>0.3666036128997803</v>
       </c>
-      <c r="H52" t="n">
+      <c r="K52" t="n">
         <v>0.08428147435188293</v>
       </c>
-      <c r="I52" t="n">
+      <c r="L52" t="n">
         <v>0.2797101449275362</v>
       </c>
-      <c r="J52" t="n">
+      <c r="M52" t="n">
         <v>5.524637681159421</v>
       </c>
-      <c r="K52" t="n">
+      <c r="N52" t="n">
         <v>6.916059865123422</v>
       </c>
-      <c r="L52" t="n">
+      <c r="O52" t="n">
         <v>0.689177749937934</v>
       </c>
-      <c r="M52" t="n">
+      <c r="P52" t="n">
         <v>0.3666036696706284</v>
       </c>
-      <c r="N52" t="n">
+      <c r="Q52" t="n">
         <v>0.6840579710144927</v>
       </c>
     </row>
@@ -2850,34 +3324,43 @@
       <c r="D53" t="n">
         <v>146</v>
       </c>
-      <c r="E53" t="b">
-        <v>1</v>
+      <c r="E53" t="n">
+        <v>82</v>
       </c>
       <c r="F53" t="n">
+        <v>39</v>
+      </c>
+      <c r="G53" t="b">
+        <v>1</v>
+      </c>
+      <c r="H53" t="n">
+        <v>118.5</v>
+      </c>
+      <c r="I53" t="n">
         <v>129</v>
       </c>
-      <c r="G53" t="n">
+      <c r="J53" t="n">
         <v>0.3826532661914825</v>
       </c>
-      <c r="H53" t="n">
+      <c r="K53" t="n">
         <v>0.08586674928665161</v>
       </c>
-      <c r="I53" t="n">
+      <c r="L53" t="n">
         <v>0.3004694835680751</v>
       </c>
-      <c r="J53" t="n">
+      <c r="M53" t="n">
         <v>5.255868544600939</v>
       </c>
-      <c r="K53" t="n">
+      <c r="N53" t="n">
         <v>6.658974435457863</v>
       </c>
-      <c r="L53" t="n">
+      <c r="O53" t="n">
         <v>0.7231252022848593</v>
       </c>
-      <c r="M53" t="n">
+      <c r="P53" t="n">
         <v>0.3826531792165496</v>
       </c>
-      <c r="N53" t="n">
+      <c r="Q53" t="n">
         <v>0.6940532081377152</v>
       </c>
     </row>
@@ -2896,34 +3379,43 @@
       <c r="D54" t="n">
         <v>150</v>
       </c>
-      <c r="E54" t="b">
-        <v>1</v>
+      <c r="E54" t="n">
+        <v>107</v>
       </c>
       <c r="F54" t="n">
+        <v>35</v>
+      </c>
+      <c r="G54" t="b">
+        <v>1</v>
+      </c>
+      <c r="H54" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="I54" t="n">
         <v>136</v>
       </c>
-      <c r="G54" t="n">
+      <c r="J54" t="n">
         <v>0.6180334687232971</v>
       </c>
-      <c r="H54" t="n">
+      <c r="K54" t="n">
         <v>0.1318826675415039</v>
       </c>
-      <c r="I54" t="n">
+      <c r="L54" t="n">
         <v>0.2936129647283127</v>
       </c>
-      <c r="J54" t="n">
+      <c r="M54" t="n">
         <v>5.763584366062917</v>
       </c>
-      <c r="K54" t="n">
+      <c r="N54" t="n">
         <v>7.681828309544007</v>
       </c>
-      <c r="L54" t="n">
+      <c r="O54" t="n">
         <v>0.5440008504636431</v>
       </c>
-      <c r="M54" t="n">
+      <c r="P54" t="n">
         <v>0.6180334612143517</v>
       </c>
-      <c r="N54" t="n">
+      <c r="Q54" t="n">
         <v>0.6391801715919924</v>
       </c>
     </row>
@@ -2942,34 +3434,43 @@
       <c r="D55" t="n">
         <v>215</v>
       </c>
-      <c r="E55" t="b">
-        <v>1</v>
+      <c r="E55" t="n">
+        <v>90</v>
       </c>
       <c r="F55" t="n">
+        <v>34</v>
+      </c>
+      <c r="G55" t="b">
+        <v>1</v>
+      </c>
+      <c r="H55" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="I55" t="n">
         <v>136</v>
       </c>
-      <c r="G55" t="n">
+      <c r="J55" t="n">
         <v>0.6598616242408752</v>
       </c>
-      <c r="H55" t="n">
+      <c r="K55" t="n">
         <v>0.01389497518539429</v>
       </c>
-      <c r="I55" t="n">
+      <c r="L55" t="n">
         <v>0.1201143946615825</v>
       </c>
-      <c r="J55" t="n">
+      <c r="M55" t="n">
         <v>12.9208770257388</v>
       </c>
-      <c r="K55" t="n">
+      <c r="N55" t="n">
         <v>16.32598097847224</v>
       </c>
-      <c r="L55" t="n">
+      <c r="O55" t="n">
         <v>0.6305052732494958</v>
       </c>
-      <c r="M55" t="n">
+      <c r="P55" t="n">
         <v>0.6598615727334606</v>
       </c>
-      <c r="N55" t="n">
+      <c r="Q55" t="n">
         <v>0.4661582459485224</v>
       </c>
     </row>
@@ -2988,34 +3489,43 @@
       <c r="D56" t="n">
         <v>140</v>
       </c>
-      <c r="E56" t="b">
-        <v>1</v>
+      <c r="E56" t="n">
+        <v>88</v>
       </c>
       <c r="F56" t="n">
+        <v>34</v>
+      </c>
+      <c r="G56" t="b">
+        <v>1</v>
+      </c>
+      <c r="H56" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="I56" t="n">
         <v>123</v>
       </c>
-      <c r="G56" t="n">
+      <c r="J56" t="n">
         <v>0.6317203640937805</v>
       </c>
-      <c r="H56" t="n">
+      <c r="K56" t="n">
         <v>0.1413600444793701</v>
       </c>
-      <c r="I56" t="n">
+      <c r="L56" t="n">
         <v>0.2610544217687075</v>
       </c>
-      <c r="J56" t="n">
+      <c r="M56" t="n">
         <v>6.216836734693878</v>
       </c>
-      <c r="K56" t="n">
+      <c r="N56" t="n">
         <v>8.144371204268944</v>
       </c>
-      <c r="L56" t="n">
+      <c r="O56" t="n">
         <v>0.6513047278496569</v>
       </c>
-      <c r="M56" t="n">
+      <c r="P56" t="n">
         <v>0.6317203476113625</v>
       </c>
-      <c r="N56" t="n">
+      <c r="Q56" t="n">
         <v>0.58078231292517</v>
       </c>
     </row>
@@ -3034,34 +3544,43 @@
       <c r="D57" t="n">
         <v>155</v>
       </c>
-      <c r="E57" t="b">
-        <v>1</v>
+      <c r="E57" t="n">
+        <v>97</v>
       </c>
       <c r="F57" t="n">
+        <v>35</v>
+      </c>
+      <c r="G57" t="b">
+        <v>1</v>
+      </c>
+      <c r="H57" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="I57" t="n">
         <v>123</v>
       </c>
-      <c r="G57" t="n">
+      <c r="J57" t="n">
         <v>0.4291980564594269</v>
       </c>
-      <c r="H57" t="n">
+      <c r="K57" t="n">
         <v>0.027080237865448</v>
       </c>
-      <c r="I57" t="n">
+      <c r="L57" t="n">
         <v>0.298686464877213</v>
       </c>
-      <c r="J57" t="n">
+      <c r="M57" t="n">
         <v>5.666476299257567</v>
       </c>
-      <c r="K57" t="n">
+      <c r="N57" t="n">
         <v>7.324415254716885</v>
       </c>
-      <c r="L57" t="n">
+      <c r="O57" t="n">
         <v>0.5480719119744413</v>
       </c>
-      <c r="M57" t="n">
+      <c r="P57" t="n">
         <v>0.4291980901256401</v>
       </c>
-      <c r="N57" t="n">
+      <c r="Q57" t="n">
         <v>0.6584808680753855</v>
       </c>
     </row>
@@ -3080,34 +3599,43 @@
       <c r="D58" t="n">
         <v>172</v>
       </c>
-      <c r="E58" t="b">
-        <v>1</v>
+      <c r="E58" t="n">
+        <v>106</v>
       </c>
       <c r="F58" t="n">
+        <v>41</v>
+      </c>
+      <c r="G58" t="b">
+        <v>1</v>
+      </c>
+      <c r="H58" t="n">
+        <v>129</v>
+      </c>
+      <c r="I58" t="n">
         <v>153</v>
       </c>
-      <c r="G58" t="n">
+      <c r="J58" t="n">
         <v>0.4619312286376953</v>
       </c>
-      <c r="H58" t="n">
+      <c r="K58" t="n">
         <v>0.1565527617931366</v>
       </c>
-      <c r="I58" t="n">
+      <c r="L58" t="n">
         <v>0.3098528756130183</v>
       </c>
-      <c r="J58" t="n">
+      <c r="M58" t="n">
         <v>5.638430673205528</v>
       </c>
-      <c r="K58" t="n">
+      <c r="N58" t="n">
         <v>7.361289745297492</v>
       </c>
-      <c r="L58" t="n">
+      <c r="O58" t="n">
         <v>0.5733502241777182</v>
       </c>
-      <c r="M58" t="n">
+      <c r="P58" t="n">
         <v>0.461931222839943</v>
       </c>
-      <c r="N58" t="n">
+      <c r="Q58" t="n">
         <v>0.7998216674097192</v>
       </c>
     </row>
@@ -3126,34 +3654,43 @@
       <c r="D59" t="n">
         <v>181</v>
       </c>
-      <c r="E59" t="b">
-        <v>1</v>
+      <c r="E59" t="n">
+        <v>99</v>
       </c>
       <c r="F59" t="n">
+        <v>41</v>
+      </c>
+      <c r="G59" t="b">
+        <v>1</v>
+      </c>
+      <c r="H59" t="n">
+        <v>129</v>
+      </c>
+      <c r="I59" t="n">
         <v>153</v>
       </c>
-      <c r="G59" t="n">
+      <c r="J59" t="n">
         <v>0.4635844230651855</v>
       </c>
-      <c r="H59" t="n">
+      <c r="K59" t="n">
         <v>0.05298137664794922</v>
       </c>
-      <c r="I59" t="n">
+      <c r="L59" t="n">
         <v>0.2858725761772853</v>
       </c>
-      <c r="J59" t="n">
+      <c r="M59" t="n">
         <v>5.938504155124654</v>
       </c>
-      <c r="K59" t="n">
+      <c r="N59" t="n">
         <v>7.683453459461566</v>
       </c>
-      <c r="L59" t="n">
+      <c r="O59" t="n">
         <v>0.5714096276990965</v>
       </c>
-      <c r="M59" t="n">
+      <c r="P59" t="n">
         <v>0.4635844688819357</v>
       </c>
-      <c r="N59" t="n">
+      <c r="Q59" t="n">
         <v>0.7601108033240997</v>
       </c>
     </row>
@@ -3172,34 +3709,43 @@
       <c r="D60" t="n">
         <v>132</v>
       </c>
-      <c r="E60" t="b">
-        <v>1</v>
+      <c r="E60" t="n">
+        <v>97</v>
       </c>
       <c r="F60" t="n">
+        <v>43</v>
+      </c>
+      <c r="G60" t="b">
+        <v>1</v>
+      </c>
+      <c r="H60" t="n">
+        <v>120.5</v>
+      </c>
+      <c r="I60" t="n">
         <v>133</v>
       </c>
-      <c r="G60" t="n">
+      <c r="J60" t="n">
         <v>0.5728060603141785</v>
       </c>
-      <c r="H60" t="n">
+      <c r="K60" t="n">
         <v>0.07629439234733582</v>
       </c>
-      <c r="I60" t="n">
+      <c r="L60" t="n">
         <v>0.2692078618225134</v>
       </c>
-      <c r="J60" t="n">
+      <c r="M60" t="n">
         <v>6.322811197141156</v>
       </c>
-      <c r="K60" t="n">
+      <c r="N60" t="n">
         <v>8.107159021337885</v>
       </c>
-      <c r="L60" t="n">
+      <c r="O60" t="n">
         <v>0.6032663518878603</v>
       </c>
-      <c r="M60" t="n">
+      <c r="P60" t="n">
         <v>0.5728060082056935</v>
       </c>
-      <c r="N60" t="n">
+      <c r="Q60" t="n">
         <v>0.6575342465753424</v>
       </c>
     </row>
@@ -3218,34 +3764,43 @@
       <c r="D61" t="n">
         <v>135</v>
       </c>
-      <c r="E61" t="b">
-        <v>1</v>
+      <c r="E61" t="n">
+        <v>106</v>
       </c>
       <c r="F61" t="n">
+        <v>42</v>
+      </c>
+      <c r="G61" t="b">
+        <v>1</v>
+      </c>
+      <c r="H61" t="n">
+        <v>120.5</v>
+      </c>
+      <c r="I61" t="n">
         <v>133</v>
       </c>
-      <c r="G61" t="n">
+      <c r="J61" t="n">
         <v>0.5297068953514099</v>
       </c>
-      <c r="H61" t="n">
+      <c r="K61" t="n">
         <v>0.1004695892333984</v>
       </c>
-      <c r="I61" t="n">
+      <c r="L61" t="n">
         <v>0.3257059396299903</v>
       </c>
-      <c r="J61" t="n">
+      <c r="M61" t="n">
         <v>5.446445959104187</v>
       </c>
-      <c r="K61" t="n">
+      <c r="N61" t="n">
         <v>7.170038004459554</v>
       </c>
-      <c r="L61" t="n">
+      <c r="O61" t="n">
         <v>0.6176143506040631</v>
       </c>
-      <c r="M61" t="n">
+      <c r="P61" t="n">
         <v>0.529706862427649</v>
       </c>
-      <c r="N61" t="n">
+      <c r="Q61" t="n">
         <v>0.6528724440116845</v>
       </c>
     </row>
@@ -3264,34 +3819,43 @@
       <c r="D62" t="n">
         <v>158</v>
       </c>
-      <c r="E62" t="b">
-        <v>1</v>
+      <c r="E62" t="n">
+        <v>95</v>
       </c>
       <c r="F62" t="n">
+        <v>39</v>
+      </c>
+      <c r="G62" t="b">
+        <v>1</v>
+      </c>
+      <c r="H62" t="n">
+        <v>125</v>
+      </c>
+      <c r="I62" t="n">
         <v>134</v>
       </c>
-      <c r="G62" t="n">
+      <c r="J62" t="n">
         <v>0.5137839913368225</v>
       </c>
-      <c r="H62" t="n">
+      <c r="K62" t="n">
         <v>0.01574355363845825</v>
       </c>
-      <c r="I62" t="n">
+      <c r="L62" t="n">
         <v>0.2300734878462408</v>
       </c>
-      <c r="J62" t="n">
+      <c r="M62" t="n">
         <v>7.003391746749576</v>
       </c>
-      <c r="K62" t="n">
+      <c r="N62" t="n">
         <v>9.005525594766114</v>
       </c>
-      <c r="L62" t="n">
+      <c r="O62" t="n">
         <v>0.5402887157566767</v>
       </c>
-      <c r="M62" t="n">
+      <c r="P62" t="n">
         <v>0.5137839054793382</v>
       </c>
-      <c r="N62" t="n">
+      <c r="Q62" t="n">
         <v>0.6613906161673262</v>
       </c>
     </row>
@@ -3310,34 +3874,43 @@
       <c r="D63" t="n">
         <v>150</v>
       </c>
-      <c r="E63" t="b">
-        <v>1</v>
+      <c r="E63" t="n">
+        <v>103</v>
       </c>
       <c r="F63" t="n">
+        <v>38</v>
+      </c>
+      <c r="G63" t="b">
+        <v>1</v>
+      </c>
+      <c r="H63" t="n">
+        <v>125</v>
+      </c>
+      <c r="I63" t="n">
         <v>134</v>
       </c>
-      <c r="G63" t="n">
+      <c r="J63" t="n">
         <v>0.5710129141807556</v>
       </c>
-      <c r="H63" t="n">
+      <c r="K63" t="n">
         <v>0.0837472677230835</v>
       </c>
-      <c r="I63" t="n">
+      <c r="L63" t="n">
         <v>0.2647554806070826</v>
       </c>
-      <c r="J63" t="n">
+      <c r="M63" t="n">
         <v>5.940978077571669</v>
       </c>
-      <c r="K63" t="n">
+      <c r="N63" t="n">
         <v>7.64865788210025</v>
       </c>
-      <c r="L63" t="n">
+      <c r="O63" t="n">
         <v>0.6134902814575941</v>
       </c>
-      <c r="M63" t="n">
+      <c r="P63" t="n">
         <v>0.571012884610769</v>
       </c>
-      <c r="N63" t="n">
+      <c r="Q63" t="n">
         <v>0.6852164137155705</v>
       </c>
     </row>
@@ -3356,34 +3929,43 @@
       <c r="D64" t="n">
         <v>133</v>
       </c>
-      <c r="E64" t="b">
-        <v>1</v>
+      <c r="E64" t="n">
+        <v>102</v>
       </c>
       <c r="F64" t="n">
+        <v>39</v>
+      </c>
+      <c r="G64" t="b">
+        <v>1</v>
+      </c>
+      <c r="H64" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="I64" t="n">
         <v>132</v>
       </c>
-      <c r="G64" t="n">
+      <c r="J64" t="n">
         <v>0.4726851582527161</v>
       </c>
-      <c r="H64" t="n">
+      <c r="K64" t="n">
         <v>0.046831876039505</v>
       </c>
-      <c r="I64" t="n">
+      <c r="L64" t="n">
         <v>0.2728551336146273</v>
       </c>
-      <c r="J64" t="n">
+      <c r="M64" t="n">
         <v>6.617440225035161</v>
       </c>
-      <c r="K64" t="n">
+      <c r="N64" t="n">
         <v>8.713763624976007</v>
       </c>
-      <c r="L64" t="n">
+      <c r="O64" t="n">
         <v>0.5794542955173515</v>
       </c>
-      <c r="M64" t="n">
+      <c r="P64" t="n">
         <v>0.4726851074789872</v>
       </c>
-      <c r="N64" t="n">
+      <c r="Q64" t="n">
         <v>0.2489451476793249</v>
       </c>
     </row>
@@ -3402,34 +3984,43 @@
       <c r="D65" t="n">
         <v>322</v>
       </c>
-      <c r="E65" t="b">
-        <v>1</v>
+      <c r="E65" t="n">
+        <v>105</v>
       </c>
       <c r="F65" t="n">
+        <v>36</v>
+      </c>
+      <c r="G65" t="b">
+        <v>1</v>
+      </c>
+      <c r="H65" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="I65" t="n">
         <v>132</v>
       </c>
-      <c r="G65" t="n">
+      <c r="J65" t="n">
         <v>0.4229510128498077</v>
       </c>
-      <c r="H65" t="n">
+      <c r="K65" t="n">
         <v>0.01764512062072754</v>
       </c>
-      <c r="I65" t="n">
+      <c r="L65" t="n">
         <v>0.2116065109695683</v>
       </c>
-      <c r="J65" t="n">
+      <c r="M65" t="n">
         <v>9.266808209483369</v>
       </c>
-      <c r="K65" t="n">
+      <c r="N65" t="n">
         <v>12.67135905933038</v>
       </c>
-      <c r="L65" t="n">
+      <c r="O65" t="n">
         <v>0.6391349646423344</v>
       </c>
-      <c r="M65" t="n">
+      <c r="P65" t="n">
         <v>0.4229510309656749</v>
       </c>
-      <c r="N65" t="n">
+      <c r="Q65" t="n">
         <v>0.2469922151450814</v>
       </c>
     </row>
@@ -3448,34 +4039,43 @@
       <c r="D66" t="n">
         <v>148</v>
       </c>
-      <c r="E66" t="b">
-        <v>1</v>
+      <c r="E66" t="n">
+        <v>96</v>
       </c>
       <c r="F66" t="n">
+        <v>40</v>
+      </c>
+      <c r="G66" t="b">
+        <v>1</v>
+      </c>
+      <c r="H66" t="n">
+        <v>119</v>
+      </c>
+      <c r="I66" t="n">
         <v>120</v>
       </c>
-      <c r="G66" t="n">
+      <c r="J66" t="n">
         <v>0.5402736663818359</v>
       </c>
-      <c r="H66" t="n">
+      <c r="K66" t="n">
         <v>0.122871607542038</v>
       </c>
-      <c r="I66" t="n">
+      <c r="L66" t="n">
         <v>0.2805999032414127</v>
       </c>
-      <c r="J66" t="n">
+      <c r="M66" t="n">
         <v>5.791969037252056</v>
       </c>
-      <c r="K66" t="n">
+      <c r="N66" t="n">
         <v>7.71674396343393</v>
       </c>
-      <c r="L66" t="n">
+      <c r="O66" t="n">
         <v>0.5359076963506563</v>
       </c>
-      <c r="M66" t="n">
+      <c r="P66" t="n">
         <v>0.5402736077895688</v>
       </c>
-      <c r="N66" t="n">
+      <c r="Q66" t="n">
         <v>0.6966618287373004</v>
       </c>
     </row>
@@ -3494,34 +4094,43 @@
       <c r="D67" t="n">
         <v>143</v>
       </c>
-      <c r="E67" t="b">
-        <v>1</v>
+      <c r="E67" t="n">
+        <v>103</v>
       </c>
       <c r="F67" t="n">
+        <v>38</v>
+      </c>
+      <c r="G67" t="b">
+        <v>1</v>
+      </c>
+      <c r="H67" t="n">
+        <v>119</v>
+      </c>
+      <c r="I67" t="n">
         <v>120</v>
       </c>
-      <c r="G67" t="n">
+      <c r="J67" t="n">
         <v>0.5208026766777039</v>
       </c>
-      <c r="H67" t="n">
+      <c r="K67" t="n">
         <v>0.08465668559074402</v>
       </c>
-      <c r="I67" t="n">
+      <c r="L67" t="n">
         <v>0.2691131498470948</v>
       </c>
-      <c r="J67" t="n">
+      <c r="M67" t="n">
         <v>6.124362895005097</v>
       </c>
-      <c r="K67" t="n">
+      <c r="N67" t="n">
         <v>8.100100048462798</v>
       </c>
-      <c r="L67" t="n">
+      <c r="O67" t="n">
         <v>0.5627717992490022</v>
       </c>
-      <c r="M67" t="n">
+      <c r="P67" t="n">
         <v>0.5208026659630685</v>
       </c>
-      <c r="N67" t="n">
+      <c r="Q67" t="n">
         <v>0.7155963302752294</v>
       </c>
     </row>
@@ -3540,34 +4149,43 @@
       <c r="D68" t="n">
         <v>162</v>
       </c>
-      <c r="E68" t="b">
-        <v>1</v>
+      <c r="E68" t="n">
+        <v>77</v>
       </c>
       <c r="F68" t="n">
+        <v>33</v>
+      </c>
+      <c r="G68" t="b">
+        <v>1</v>
+      </c>
+      <c r="H68" t="n">
+        <v>124</v>
+      </c>
+      <c r="I68" t="n">
         <v>148</v>
       </c>
-      <c r="G68" t="n">
+      <c r="J68" t="n">
         <v>0.6092353463172913</v>
       </c>
-      <c r="H68" t="n">
+      <c r="K68" t="n">
         <v>0.1955194771289825</v>
       </c>
-      <c r="I68" t="n">
+      <c r="L68" t="n">
         <v>0.253968253968254</v>
       </c>
-      <c r="J68" t="n">
+      <c r="M68" t="n">
         <v>6.634920634920635</v>
       </c>
-      <c r="K68" t="n">
+      <c r="N68" t="n">
         <v>8.584645893961879</v>
       </c>
-      <c r="L68" t="n">
+      <c r="O68" t="n">
         <v>0.609360553485778</v>
       </c>
-      <c r="M68" t="n">
+      <c r="P68" t="n">
         <v>0.6092353598272308</v>
       </c>
-      <c r="N68" t="n">
+      <c r="Q68" t="n">
         <v>0.6167800453514739</v>
       </c>
     </row>
@@ -3586,34 +4204,43 @@
       <c r="D69" t="n">
         <v>160</v>
       </c>
-      <c r="E69" t="b">
-        <v>1</v>
+      <c r="E69" t="n">
+        <v>79</v>
       </c>
       <c r="F69" t="n">
+        <v>35</v>
+      </c>
+      <c r="G69" t="b">
+        <v>1</v>
+      </c>
+      <c r="H69" t="n">
+        <v>124</v>
+      </c>
+      <c r="I69" t="n">
         <v>148</v>
       </c>
-      <c r="G69" t="n">
+      <c r="J69" t="n">
         <v>0.5944502353668213</v>
       </c>
-      <c r="H69" t="n">
+      <c r="K69" t="n">
         <v>0.09678319096565247</v>
       </c>
-      <c r="I69" t="n">
+      <c r="L69" t="n">
         <v>0.2788732394366197</v>
       </c>
-      <c r="J69" t="n">
+      <c r="M69" t="n">
         <v>6.836619718309859</v>
       </c>
-      <c r="K69" t="n">
+      <c r="N69" t="n">
         <v>9.139914013217744</v>
       </c>
-      <c r="L69" t="n">
+      <c r="O69" t="n">
         <v>0.6150618976472976</v>
       </c>
-      <c r="M69" t="n">
+      <c r="P69" t="n">
         <v>0.5944502192655898</v>
       </c>
-      <c r="N69" t="n">
+      <c r="Q69" t="n">
         <v>0.5725352112676056</v>
       </c>
     </row>
@@ -3632,34 +4259,43 @@
       <c r="D70" t="n">
         <v>175</v>
       </c>
-      <c r="E70" t="b">
-        <v>1</v>
+      <c r="E70" t="n">
+        <v>109</v>
       </c>
       <c r="F70" t="n">
+        <v>45</v>
+      </c>
+      <c r="G70" t="b">
+        <v>1</v>
+      </c>
+      <c r="H70" t="n">
+        <v>138</v>
+      </c>
+      <c r="I70" t="n">
         <v>171</v>
       </c>
-      <c r="G70" t="n">
+      <c r="J70" t="n">
         <v>0.5220439434051514</v>
       </c>
-      <c r="H70" t="n">
+      <c r="K70" t="n">
         <v>0.1366487145423889</v>
       </c>
-      <c r="I70" t="n">
+      <c r="L70" t="n">
         <v>0.2808219178082192</v>
       </c>
-      <c r="J70" t="n">
+      <c r="M70" t="n">
         <v>5.886806056236481</v>
       </c>
-      <c r="K70" t="n">
+      <c r="N70" t="n">
         <v>7.762331167104442</v>
       </c>
-      <c r="L70" t="n">
+      <c r="O70" t="n">
         <v>0.56210931987584</v>
       </c>
-      <c r="M70" t="n">
+      <c r="P70" t="n">
         <v>0.5220438957175644</v>
       </c>
-      <c r="N70" t="n">
+      <c r="Q70" t="n">
         <v>0.5739005046863734</v>
       </c>
     </row>
@@ -3678,34 +4314,43 @@
       <c r="D71" t="n">
         <v>212</v>
       </c>
-      <c r="E71" t="b">
-        <v>1</v>
+      <c r="E71" t="n">
+        <v>94</v>
       </c>
       <c r="F71" t="n">
+        <v>61</v>
+      </c>
+      <c r="G71" t="b">
+        <v>1</v>
+      </c>
+      <c r="H71" t="n">
+        <v>138</v>
+      </c>
+      <c r="I71" t="n">
         <v>171</v>
       </c>
-      <c r="G71" t="n">
+      <c r="J71" t="n">
         <v>0.471458375453949</v>
       </c>
-      <c r="H71" t="n">
+      <c r="K71" t="n">
         <v>0.0421503484249115</v>
       </c>
-      <c r="I71" t="n">
+      <c r="L71" t="n">
         <v>0.2056737588652482</v>
       </c>
-      <c r="J71" t="n">
+      <c r="M71" t="n">
         <v>8.254643701452212</v>
       </c>
-      <c r="K71" t="n">
+      <c r="N71" t="n">
         <v>10.67492714593832</v>
       </c>
-      <c r="L71" t="n">
+      <c r="O71" t="n">
         <v>0.5203453045177235</v>
       </c>
-      <c r="M71" t="n">
+      <c r="P71" t="n">
         <v>0.4714583178550396</v>
       </c>
-      <c r="N71" t="n">
+      <c r="Q71" t="n">
         <v>0.4380276933468423</v>
       </c>
     </row>
@@ -3724,34 +4369,43 @@
       <c r="D72" t="n">
         <v>145</v>
       </c>
-      <c r="E72" t="b">
-        <v>1</v>
+      <c r="E72" t="n">
+        <v>73</v>
       </c>
       <c r="F72" t="n">
+        <v>35</v>
+      </c>
+      <c r="G72" t="b">
+        <v>1</v>
+      </c>
+      <c r="H72" t="n">
+        <v>123</v>
+      </c>
+      <c r="I72" t="n">
         <v>116</v>
       </c>
-      <c r="G72" t="n">
+      <c r="J72" t="n">
         <v>0.6825814843177795</v>
       </c>
-      <c r="H72" t="n">
+      <c r="K72" t="n">
         <v>0.03291523456573486</v>
       </c>
-      <c r="I72" t="n">
+      <c r="L72" t="n">
         <v>0.177319587628866</v>
       </c>
-      <c r="J72" t="n">
+      <c r="M72" t="n">
         <v>8.102061855670103</v>
       </c>
-      <c r="K72" t="n">
+      <c r="N72" t="n">
         <v>10.24830888739925</v>
       </c>
-      <c r="L72" t="n">
+      <c r="O72" t="n">
         <v>0.6172867066759036</v>
       </c>
-      <c r="M72" t="n">
+      <c r="P72" t="n">
         <v>0.682581454531703</v>
       </c>
-      <c r="N72" t="n">
+      <c r="Q72" t="n">
         <v>0.5845360824742268</v>
       </c>
     </row>
@@ -3770,34 +4424,43 @@
       <c r="D73" t="n">
         <v>129</v>
       </c>
-      <c r="E73" t="b">
-        <v>1</v>
+      <c r="E73" t="n">
+        <v>98</v>
       </c>
       <c r="F73" t="n">
+        <v>37</v>
+      </c>
+      <c r="G73" t="b">
+        <v>1</v>
+      </c>
+      <c r="H73" t="n">
+        <v>123</v>
+      </c>
+      <c r="I73" t="n">
         <v>116</v>
       </c>
-      <c r="G73" t="n">
+      <c r="J73" t="n">
         <v>0.6543575525283813</v>
       </c>
-      <c r="H73" t="n">
+      <c r="K73" t="n">
         <v>0.1218281388282776</v>
       </c>
-      <c r="I73" t="n">
+      <c r="L73" t="n">
         <v>0.2322456813819578</v>
       </c>
-      <c r="J73" t="n">
+      <c r="M73" t="n">
         <v>7.50911708253359</v>
       </c>
-      <c r="K73" t="n">
+      <c r="N73" t="n">
         <v>9.899034443695324</v>
       </c>
-      <c r="L73" t="n">
+      <c r="O73" t="n">
         <v>0.5791275803313773</v>
       </c>
-      <c r="M73" t="n">
+      <c r="P73" t="n">
         <v>0.6543576895265767</v>
       </c>
-      <c r="N73" t="n">
+      <c r="Q73" t="n">
         <v>0.6650671785028791</v>
       </c>
     </row>
@@ -3816,34 +4479,43 @@
       <c r="D74" t="n">
         <v>236</v>
       </c>
-      <c r="E74" t="b">
-        <v>1</v>
+      <c r="E74" t="n">
+        <v>75</v>
       </c>
       <c r="F74" t="n">
+        <v>30</v>
+      </c>
+      <c r="G74" t="b">
+        <v>1</v>
+      </c>
+      <c r="H74" t="n">
+        <v>125.5</v>
+      </c>
+      <c r="I74" t="n">
         <v>97</v>
       </c>
-      <c r="G74" t="n">
+      <c r="J74" t="n">
         <v>0.691866934299469</v>
       </c>
-      <c r="H74" t="n">
+      <c r="K74" t="n">
         <v>0.09595531225204468</v>
       </c>
-      <c r="I74" t="n">
+      <c r="L74" t="n">
         <v>0.09014084507042254</v>
       </c>
-      <c r="J74" t="n">
+      <c r="M74" t="n">
         <v>30.11830985915493</v>
       </c>
-      <c r="K74" t="n">
+      <c r="N74" t="n">
         <v>56.82029988369684</v>
       </c>
-      <c r="L74" t="n">
+      <c r="O74" t="n">
         <v>0.808849705174841</v>
       </c>
-      <c r="M74" t="n">
+      <c r="P74" t="n">
         <v>0.691866949512509</v>
       </c>
-      <c r="N74" t="n">
+      <c r="Q74" t="n">
         <v>0.2338028169014084</v>
       </c>
     </row>
@@ -3862,34 +4534,43 @@
       <c r="D75" t="n">
         <v>101</v>
       </c>
-      <c r="E75" t="b">
-        <v>1</v>
+      <c r="E75" t="n">
+        <v>91</v>
       </c>
       <c r="F75" t="n">
+        <v>31</v>
+      </c>
+      <c r="G75" t="b">
+        <v>1</v>
+      </c>
+      <c r="H75" t="n">
+        <v>125.5</v>
+      </c>
+      <c r="I75" t="n">
         <v>97</v>
       </c>
-      <c r="G75" t="n">
+      <c r="J75" t="n">
         <v>0.5278096795082092</v>
       </c>
-      <c r="H75" t="n">
+      <c r="K75" t="n">
         <v>0.04484131932258606</v>
       </c>
-      <c r="I75" t="n">
+      <c r="L75" t="n">
         <v>0.1680790960451977</v>
       </c>
-      <c r="J75" t="n">
+      <c r="M75" t="n">
         <v>9.861581920903955</v>
       </c>
-      <c r="K75" t="n">
+      <c r="N75" t="n">
         <v>12.08725340659549</v>
       </c>
-      <c r="L75" t="n">
+      <c r="O75" t="n">
         <v>0.6828829980727591</v>
       </c>
-      <c r="M75" t="n">
+      <c r="P75" t="n">
         <v>0.5278096870056965</v>
       </c>
-      <c r="N75" t="n">
+      <c r="Q75" t="n">
         <v>0.5734463276836158</v>
       </c>
     </row>
@@ -3908,34 +4589,43 @@
       <c r="D76" t="n">
         <v>137</v>
       </c>
-      <c r="E76" t="b">
-        <v>1</v>
+      <c r="E76" t="n">
+        <v>105</v>
       </c>
       <c r="F76" t="n">
+        <v>39</v>
+      </c>
+      <c r="G76" t="b">
+        <v>1</v>
+      </c>
+      <c r="H76" t="n">
+        <v>127</v>
+      </c>
+      <c r="I76" t="n">
         <v>130</v>
       </c>
-      <c r="G76" t="n">
+      <c r="J76" t="n">
         <v>0.5923114418983459</v>
       </c>
-      <c r="H76" t="n">
+      <c r="K76" t="n">
         <v>0.171817421913147</v>
       </c>
-      <c r="I76" t="n">
+      <c r="L76" t="n">
         <v>0.276707530647986</v>
       </c>
-      <c r="J76" t="n">
+      <c r="M76" t="n">
         <v>6.18739054290718</v>
       </c>
-      <c r="K76" t="n">
+      <c r="N76" t="n">
         <v>8.361609936123321</v>
       </c>
-      <c r="L76" t="n">
+      <c r="O76" t="n">
         <v>0.5961926863440321</v>
       </c>
-      <c r="M76" t="n">
+      <c r="P76" t="n">
         <v>0.5923114233111778</v>
       </c>
-      <c r="N76" t="n">
+      <c r="Q76" t="n">
         <v>0.7472270869819031</v>
       </c>
     </row>
@@ -3954,34 +4644,43 @@
       <c r="D77" t="n">
         <v>175</v>
       </c>
-      <c r="E77" t="b">
-        <v>1</v>
+      <c r="E77" t="n">
+        <v>100</v>
       </c>
       <c r="F77" t="n">
+        <v>43</v>
+      </c>
+      <c r="G77" t="b">
+        <v>1</v>
+      </c>
+      <c r="H77" t="n">
+        <v>127</v>
+      </c>
+      <c r="I77" t="n">
         <v>130</v>
       </c>
-      <c r="G77" t="n">
+      <c r="J77" t="n">
         <v>0.5268495678901672</v>
       </c>
-      <c r="H77" t="n">
+      <c r="K77" t="n">
         <v>0.1398022770881653</v>
       </c>
-      <c r="I77" t="n">
+      <c r="L77" t="n">
         <v>0.2875189489641233</v>
       </c>
-      <c r="J77" t="n">
+      <c r="M77" t="n">
         <v>5.332491157150076</v>
       </c>
-      <c r="K77" t="n">
+      <c r="N77" t="n">
         <v>6.892482594927204</v>
       </c>
-      <c r="L77" t="n">
+      <c r="O77" t="n">
         <v>0.5049349825175882</v>
       </c>
-      <c r="M77" t="n">
+      <c r="P77" t="n">
         <v>0.5268496187176555</v>
       </c>
-      <c r="N77" t="n">
+      <c r="Q77" t="n">
         <v>0.7569479535118747</v>
       </c>
     </row>
@@ -4000,34 +4699,43 @@
       <c r="D78" t="n">
         <v>125</v>
       </c>
-      <c r="E78" t="b">
-        <v>1</v>
+      <c r="E78" t="n">
+        <v>99</v>
       </c>
       <c r="F78" t="n">
+        <v>33</v>
+      </c>
+      <c r="G78" t="b">
+        <v>1</v>
+      </c>
+      <c r="H78" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="I78" t="n">
         <v>129</v>
       </c>
-      <c r="G78" t="n">
+      <c r="J78" t="n">
         <v>0.6168738603591919</v>
       </c>
-      <c r="H78" t="n">
+      <c r="K78" t="n">
         <v>0.11076420545578</v>
       </c>
-      <c r="I78" t="n">
+      <c r="L78" t="n">
         <v>0.2125356125356125</v>
       </c>
-      <c r="J78" t="n">
+      <c r="M78" t="n">
         <v>9.697435897435897</v>
       </c>
-      <c r="K78" t="n">
+      <c r="N78" t="n">
         <v>13.0941147259309</v>
       </c>
-      <c r="L78" t="n">
+      <c r="O78" t="n">
         <v>0.5170628123132698</v>
       </c>
-      <c r="M78" t="n">
+      <c r="P78" t="n">
         <v>0.6168738433720536</v>
       </c>
-      <c r="N78" t="n">
+      <c r="Q78" t="n">
         <v>0.7834757834757835</v>
       </c>
     </row>
@@ -4046,34 +4754,43 @@
       <c r="D79" t="n">
         <v>143</v>
       </c>
-      <c r="E79" t="b">
-        <v>1</v>
+      <c r="E79" t="n">
+        <v>87</v>
       </c>
       <c r="F79" t="n">
+        <v>34</v>
+      </c>
+      <c r="G79" t="b">
+        <v>1</v>
+      </c>
+      <c r="H79" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="I79" t="n">
         <v>129</v>
       </c>
-      <c r="G79" t="n">
+      <c r="J79" t="n">
         <v>0.6988266706466675</v>
       </c>
-      <c r="H79" t="n">
+      <c r="K79" t="n">
         <v>0.1308326721191406</v>
       </c>
-      <c r="I79" t="n">
+      <c r="L79" t="n">
         <v>0.2287581699346405</v>
       </c>
-      <c r="J79" t="n">
+      <c r="M79" t="n">
         <v>7.458333333333333</v>
       </c>
-      <c r="K79" t="n">
+      <c r="N79" t="n">
         <v>10.03486568977207</v>
       </c>
-      <c r="L79" t="n">
+      <c r="O79" t="n">
         <v>0.5962869602977243</v>
       </c>
-      <c r="M79" t="n">
+      <c r="P79" t="n">
         <v>0.6988266318715779</v>
       </c>
-      <c r="N79" t="n">
+      <c r="Q79" t="n">
         <v>0.7516339869281046</v>
       </c>
     </row>
@@ -4092,34 +4809,43 @@
       <c r="D80" t="n">
         <v>127</v>
       </c>
-      <c r="E80" t="b">
-        <v>1</v>
+      <c r="E80" t="n">
+        <v>84</v>
       </c>
       <c r="F80" t="n">
+        <v>33</v>
+      </c>
+      <c r="G80" t="b">
+        <v>1</v>
+      </c>
+      <c r="H80" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="I80" t="n">
         <v>106</v>
       </c>
-      <c r="G80" t="n">
+      <c r="J80" t="n">
         <v>0.6140279173851013</v>
       </c>
-      <c r="H80" t="n">
+      <c r="K80" t="n">
         <v>0.1769627630710602</v>
       </c>
-      <c r="I80" t="n">
+      <c r="L80" t="n">
         <v>0.2342819324950364</v>
       </c>
-      <c r="J80" t="n">
+      <c r="M80" t="n">
         <v>6.902713434811383</v>
       </c>
-      <c r="K80" t="n">
+      <c r="N80" t="n">
         <v>9.090616685027294</v>
       </c>
-      <c r="L80" t="n">
+      <c r="O80" t="n">
         <v>0.5940135081775652</v>
       </c>
-      <c r="M80" t="n">
+      <c r="P80" t="n">
         <v>0.6140279561428471</v>
       </c>
-      <c r="N80" t="n">
+      <c r="Q80" t="n">
         <v>0.6201191264063534</v>
       </c>
     </row>
@@ -4138,34 +4864,43 @@
       <c r="D81" t="n">
         <v>131</v>
       </c>
-      <c r="E81" t="b">
-        <v>1</v>
+      <c r="E81" t="n">
+        <v>85</v>
       </c>
       <c r="F81" t="n">
+        <v>33</v>
+      </c>
+      <c r="G81" t="b">
+        <v>1</v>
+      </c>
+      <c r="H81" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="I81" t="n">
         <v>106</v>
       </c>
-      <c r="G81" t="n">
+      <c r="J81" t="n">
         <v>0.606816291809082</v>
       </c>
-      <c r="H81" t="n">
+      <c r="K81" t="n">
         <v>0.1125555336475372</v>
       </c>
-      <c r="I81" t="n">
+      <c r="L81" t="n">
         <v>0.2423378474697078</v>
       </c>
-      <c r="J81" t="n">
+      <c r="M81" t="n">
         <v>6.414825374198147</v>
       </c>
-      <c r="K81" t="n">
+      <c r="N81" t="n">
         <v>8.256231582446034</v>
       </c>
-      <c r="L81" t="n">
+      <c r="O81" t="n">
         <v>0.5923615099468964</v>
       </c>
-      <c r="M81" t="n">
+      <c r="P81" t="n">
         <v>0.6068163675164767</v>
       </c>
-      <c r="N81" t="n">
+      <c r="Q81" t="n">
         <v>0.6037063435495367</v>
       </c>
     </row>

</xml_diff>